<commit_message>
inside bbo, min tick
</commit_message>
<xml_diff>
--- a/sheets/fill_stats.xlsx
+++ b/sheets/fill_stats.xlsx
@@ -486,31 +486,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>47.5</v>
+        <v>25.6</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="D3" t="n">
-        <v>51.7</v>
+        <v>73.5</v>
       </c>
       <c r="E3" t="n">
-        <v>0.959</v>
+        <v>0.52</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0123</v>
+        <v>0.0264</v>
       </c>
       <c r="G3" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0174</v>
       </c>
       <c r="H3" t="n">
-        <v>53.5</v>
+        <v>50.5</v>
       </c>
       <c r="I3" t="n">
-        <v>22.7</v>
+        <v>23.2</v>
       </c>
       <c r="J3" t="n">
-        <v>23.8</v>
+        <v>26.3</v>
       </c>
     </row>
     <row r="4">
@@ -520,31 +520,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>25</v>
+        <v>8.1</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>74.90000000000001</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>0.501</v>
+        <v>0.162</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0129</v>
+        <v>0.0526</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0021</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>53.4</v>
+        <v>64.8</v>
       </c>
       <c r="I4" t="n">
-        <v>42.8</v>
+        <v>31.1</v>
       </c>
       <c r="J4" t="n">
-        <v>3.7</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="5">
@@ -554,31 +554,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>73.90000000000001</v>
+        <v>47.6</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4</v>
+        <v>2.5</v>
       </c>
       <c r="D5" t="n">
-        <v>25.8</v>
+        <v>49.9</v>
       </c>
       <c r="E5" t="n">
-        <v>1.482</v>
+        <v>0.977</v>
       </c>
       <c r="F5" t="n">
-        <v>0.019</v>
+        <v>0.0169</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0024</v>
+        <v>0.0258</v>
       </c>
       <c r="H5" t="n">
-        <v>19.8</v>
+        <v>38.6</v>
       </c>
       <c r="I5" t="n">
-        <v>76.8</v>
+        <v>54.5</v>
       </c>
       <c r="J5" t="n">
-        <v>3.3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -588,31 +588,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>56.6</v>
+        <v>25.2</v>
       </c>
       <c r="C6" t="n">
-        <v>0.1</v>
+        <v>1.8</v>
       </c>
       <c r="D6" t="n">
-        <v>43.4</v>
+        <v>73</v>
       </c>
       <c r="E6" t="n">
-        <v>1.132</v>
+        <v>0.522</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0151</v>
+        <v>0.0251</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0347</v>
       </c>
       <c r="H6" t="n">
-        <v>30.4</v>
+        <v>45.8</v>
       </c>
       <c r="I6" t="n">
-        <v>66.3</v>
+        <v>51</v>
       </c>
       <c r="J6" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="10">
@@ -681,31 +681,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>22.5</v>
+        <v>9</v>
       </c>
       <c r="C12" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="D12" t="n">
-        <v>76.59999999999999</v>
+        <v>89.8</v>
       </c>
       <c r="E12" t="n">
-        <v>0.458</v>
+        <v>0.193</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0104</v>
+        <v>0.0184</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0195</v>
+        <v>0.0617</v>
       </c>
       <c r="H12" t="n">
-        <v>43.7</v>
+        <v>46.8</v>
       </c>
       <c r="I12" t="n">
-        <v>24.7</v>
+        <v>18.3</v>
       </c>
       <c r="J12" t="n">
-        <v>31.6</v>
+        <v>34.9</v>
       </c>
     </row>
     <row r="13">
@@ -715,31 +715,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>8.6</v>
+        <v>1.4</v>
       </c>
       <c r="C13" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="D13" t="n">
-        <v>91</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="E13" t="n">
-        <v>0.176</v>
+        <v>0.03</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0173</v>
+        <v>0.0314</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0209</v>
+        <v>0.0801</v>
       </c>
       <c r="H13" t="n">
-        <v>31.8</v>
+        <v>70.3</v>
       </c>
       <c r="I13" t="n">
-        <v>64</v>
+        <v>27.3</v>
       </c>
       <c r="J13" t="n">
-        <v>4.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="14">
@@ -749,31 +749,31 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>58</v>
+        <v>29.8</v>
       </c>
       <c r="C14" t="n">
-        <v>1.3</v>
+        <v>1.5</v>
       </c>
       <c r="D14" t="n">
-        <v>40.6</v>
+        <v>68.7</v>
       </c>
       <c r="E14" t="n">
-        <v>1.174</v>
+        <v>0.611</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0103</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0114</v>
+        <v>0.0244</v>
       </c>
       <c r="H14" t="n">
-        <v>22.2</v>
+        <v>43.5</v>
       </c>
       <c r="I14" t="n">
-        <v>75.40000000000001</v>
+        <v>52.3</v>
       </c>
       <c r="J14" t="n">
-        <v>2.4</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="15">
@@ -783,31 +783,31 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>35.1</v>
+        <v>12.4</v>
       </c>
       <c r="C15" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>64.59999999999999</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="E15" t="n">
-        <v>0.705</v>
+        <v>0.258</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0048</v>
+        <v>-0.0016</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0036</v>
+        <v>0.0381</v>
       </c>
       <c r="H15" t="n">
-        <v>35.4</v>
+        <v>50.4</v>
       </c>
       <c r="I15" t="n">
-        <v>62.1</v>
+        <v>48.2</v>
       </c>
       <c r="J15" t="n">
-        <v>2.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="19">
@@ -876,31 +876,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>26</v>
+        <v>10.7</v>
       </c>
       <c r="C21" t="n">
-        <v>0.4</v>
+        <v>1.5</v>
       </c>
       <c r="D21" t="n">
-        <v>73.59999999999999</v>
+        <v>87.8</v>
       </c>
       <c r="E21" t="n">
-        <v>0.525</v>
+        <v>0.229</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.0012</v>
+        <v>0.0375</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0081</v>
+        <v>0.0673</v>
       </c>
       <c r="H21" t="n">
-        <v>45.7</v>
+        <v>48.5</v>
       </c>
       <c r="I21" t="n">
-        <v>24.4</v>
+        <v>15.9</v>
       </c>
       <c r="J21" t="n">
-        <v>29.9</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="22">
@@ -910,31 +910,31 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>10.2</v>
+        <v>1.5</v>
       </c>
       <c r="C22" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="D22" t="n">
-        <v>89.5</v>
+        <v>98.3</v>
       </c>
       <c r="E22" t="n">
-        <v>0.207</v>
+        <v>0.032</v>
       </c>
       <c r="F22" t="n">
-        <v>0.0043</v>
+        <v>-0.07829999999999999</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0144</v>
+        <v>0.0592</v>
       </c>
       <c r="H22" t="n">
-        <v>34.3</v>
+        <v>78</v>
       </c>
       <c r="I22" t="n">
-        <v>62</v>
+        <v>21.1</v>
       </c>
       <c r="J22" t="n">
-        <v>3.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="23">
@@ -944,31 +944,31 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>57.9</v>
+        <v>31</v>
       </c>
       <c r="C23" t="n">
-        <v>0.7</v>
+        <v>1.4</v>
       </c>
       <c r="D23" t="n">
-        <v>41.4</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="E23" t="n">
-        <v>1.166</v>
+        <v>0.634</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0102</v>
+        <v>0.0366</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0061</v>
+        <v>0.0213</v>
       </c>
       <c r="H23" t="n">
-        <v>24.5</v>
+        <v>44.8</v>
       </c>
       <c r="I23" t="n">
-        <v>73</v>
+        <v>50.5</v>
       </c>
       <c r="J23" t="n">
-        <v>2.5</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="24">
@@ -978,31 +978,31 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>36</v>
+        <v>13.1</v>
       </c>
       <c r="C24" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="D24" t="n">
-        <v>63.5</v>
+        <v>85.5</v>
       </c>
       <c r="E24" t="n">
-        <v>0.725</v>
+        <v>0.276</v>
       </c>
       <c r="F24" t="n">
-        <v>-0.0038</v>
+        <v>-0.0064</v>
       </c>
       <c r="G24" t="n">
-        <v>0.0073</v>
+        <v>0.0526</v>
       </c>
       <c r="H24" t="n">
-        <v>35.3</v>
+        <v>51.6</v>
       </c>
       <c r="I24" t="n">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="J24" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="28">
@@ -1071,31 +1071,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>22.3</v>
+        <v>10</v>
       </c>
       <c r="C30" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="D30" t="n">
-        <v>77.5</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="E30" t="n">
-        <v>0.448</v>
+        <v>0.204</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.0113</v>
+        <v>0.004</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0044</v>
+        <v>0.0218</v>
       </c>
       <c r="H30" t="n">
-        <v>45.3</v>
+        <v>48.9</v>
       </c>
       <c r="I30" t="n">
-        <v>20.6</v>
+        <v>19.1</v>
       </c>
       <c r="J30" t="n">
-        <v>34.2</v>
+        <v>32.1</v>
       </c>
     </row>
     <row r="31">
@@ -1105,31 +1105,31 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>7.7</v>
+        <v>1.6</v>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D31" t="n">
-        <v>92.3</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="E31" t="n">
-        <v>0.154</v>
+        <v>0.035</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.023</v>
+        <v>0.0171</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0025</v>
+        <v>0.0718</v>
       </c>
       <c r="H31" t="n">
-        <v>35.9</v>
+        <v>73.8</v>
       </c>
       <c r="I31" t="n">
-        <v>59.9</v>
+        <v>25.1</v>
       </c>
       <c r="J31" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -1139,31 +1139,31 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>58.5</v>
+        <v>30.6</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D32" t="n">
-        <v>39.5</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="E32" t="n">
-        <v>1.189</v>
+        <v>0.642</v>
       </c>
       <c r="F32" t="n">
-        <v>0.0026</v>
+        <v>0.0136</v>
       </c>
       <c r="G32" t="n">
-        <v>0.0168</v>
+        <v>0.046</v>
       </c>
       <c r="H32" t="n">
-        <v>21.7</v>
+        <v>43.5</v>
       </c>
       <c r="I32" t="n">
-        <v>75.7</v>
+        <v>52.5</v>
       </c>
       <c r="J32" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="33">
@@ -1173,31 +1173,31 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>34.5</v>
+        <v>12.3</v>
       </c>
       <c r="C33" t="n">
-        <v>3.6</v>
+        <v>2.1</v>
       </c>
       <c r="D33" t="n">
-        <v>61.8</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="E33" t="n">
-        <v>0.727</v>
+        <v>0.267</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0057</v>
+        <v>0.0244</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0496</v>
+        <v>0.0789</v>
       </c>
       <c r="H33" t="n">
-        <v>35.4</v>
+        <v>50.1</v>
       </c>
       <c r="I33" t="n">
-        <v>62.4</v>
+        <v>48.2</v>
       </c>
       <c r="J33" t="n">
-        <v>2.2</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="37">
@@ -1266,31 +1266,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>17.9</v>
+        <v>7.9</v>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="D39" t="n">
-        <v>81.09999999999999</v>
+        <v>90.8</v>
       </c>
       <c r="E39" t="n">
-        <v>0.369</v>
+        <v>0.172</v>
       </c>
       <c r="F39" t="n">
-        <v>0.0223</v>
+        <v>0.0212</v>
       </c>
       <c r="G39" t="n">
-        <v>0.0264</v>
+        <v>0.0764</v>
       </c>
       <c r="H39" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I39" t="n">
-        <v>16.3</v>
+        <v>17.6</v>
       </c>
       <c r="J39" t="n">
-        <v>37.7</v>
+        <v>34.5</v>
       </c>
     </row>
     <row r="40">
@@ -1300,31 +1300,31 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>5</v>
+        <v>0.9</v>
       </c>
       <c r="C40" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="D40" t="n">
-        <v>94.7</v>
+        <v>98.7</v>
       </c>
       <c r="E40" t="n">
-        <v>0.103</v>
+        <v>0.022</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0027</v>
+        <v>-0.025</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0293</v>
+        <v>0.1592</v>
       </c>
       <c r="H40" t="n">
-        <v>34.1</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="I40" t="n">
-        <v>62.1</v>
+        <v>22.9</v>
       </c>
       <c r="J40" t="n">
-        <v>3.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1334,31 +1334,31 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>57.5</v>
+        <v>28.7</v>
       </c>
       <c r="C41" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="D41" t="n">
-        <v>41.8</v>
+        <v>70.8</v>
       </c>
       <c r="E41" t="n">
-        <v>1.156</v>
+        <v>0.578</v>
       </c>
       <c r="F41" t="n">
-        <v>0.0086</v>
+        <v>-0.0117</v>
       </c>
       <c r="G41" t="n">
-        <v>0.006</v>
+        <v>0.0089</v>
       </c>
       <c r="H41" t="n">
-        <v>20.4</v>
+        <v>43.1</v>
       </c>
       <c r="I41" t="n">
-        <v>77.5</v>
+        <v>52.9</v>
       </c>
       <c r="J41" t="n">
-        <v>2.1</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="42">
@@ -1368,31 +1368,31 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>32.1</v>
+        <v>11.5</v>
       </c>
       <c r="C42" t="n">
-        <v>2.5</v>
+        <v>1.6</v>
       </c>
       <c r="D42" t="n">
-        <v>65.5</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="E42" t="n">
-        <v>0.666</v>
+        <v>0.247</v>
       </c>
       <c r="F42" t="n">
-        <v>0.0127</v>
+        <v>-0.0019</v>
       </c>
       <c r="G42" t="n">
-        <v>0.037</v>
+        <v>0.0644</v>
       </c>
       <c r="H42" t="n">
-        <v>34.5</v>
+        <v>49.9</v>
       </c>
       <c r="I42" t="n">
-        <v>63.5</v>
+        <v>48.4</v>
       </c>
       <c r="J42" t="n">
-        <v>2</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="46">
@@ -1461,31 +1461,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>27.3</v>
+        <v>12.6</v>
       </c>
       <c r="C48" t="n">
-        <v>0.7</v>
+        <v>1.1</v>
       </c>
       <c r="D48" t="n">
-        <v>72.09999999999999</v>
+        <v>86.3</v>
       </c>
       <c r="E48" t="n">
-        <v>0.552</v>
+        <v>0.264</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0065</v>
+        <v>0.0215</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0134</v>
+        <v>0.0489</v>
       </c>
       <c r="H48" t="n">
-        <v>48</v>
+        <v>48.9</v>
       </c>
       <c r="I48" t="n">
-        <v>22.1</v>
+        <v>19.6</v>
       </c>
       <c r="J48" t="n">
-        <v>29.9</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="49">
@@ -1495,31 +1495,31 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>11.3</v>
+        <v>2.7</v>
       </c>
       <c r="C49" t="n">
         <v>0.2</v>
       </c>
       <c r="D49" t="n">
-        <v>88.5</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="E49" t="n">
-        <v>0.228</v>
+        <v>0.056</v>
       </c>
       <c r="F49" t="n">
-        <v>0.0028</v>
+        <v>-0.0004</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0139</v>
+        <v>0.0741</v>
       </c>
       <c r="H49" t="n">
-        <v>42.3</v>
+        <v>69.2</v>
       </c>
       <c r="I49" t="n">
-        <v>53.8</v>
+        <v>28</v>
       </c>
       <c r="J49" t="n">
-        <v>3.9</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="50">
@@ -1529,31 +1529,31 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>61.2</v>
+        <v>33.5</v>
       </c>
       <c r="C50" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="D50" t="n">
-        <v>37.8</v>
+        <v>64.7</v>
       </c>
       <c r="E50" t="n">
-        <v>1.233</v>
+        <v>0.6879999999999999</v>
       </c>
       <c r="F50" t="n">
-        <v>0.0101</v>
+        <v>0.0111</v>
       </c>
       <c r="G50" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0253</v>
       </c>
       <c r="H50" t="n">
-        <v>21.6</v>
+        <v>42.3</v>
       </c>
       <c r="I50" t="n">
-        <v>75.8</v>
+        <v>52.7</v>
       </c>
       <c r="J50" t="n">
-        <v>2.6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51">
@@ -1563,31 +1563,31 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>38.9</v>
+        <v>14.9</v>
       </c>
       <c r="C51" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
       <c r="D51" t="n">
-        <v>59.8</v>
+        <v>83.5</v>
       </c>
       <c r="E51" t="n">
-        <v>0.791</v>
+        <v>0.314</v>
       </c>
       <c r="F51" t="n">
-        <v>0.005</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="G51" t="n">
-        <v>0.0196</v>
+        <v>0.0537</v>
       </c>
       <c r="H51" t="n">
-        <v>33.8</v>
+        <v>49.1</v>
       </c>
       <c r="I51" t="n">
-        <v>63.6</v>
+        <v>48.6</v>
       </c>
       <c r="J51" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
     </row>
   </sheetData>
@@ -1670,31 +1670,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>12.5</v>
+        <v>10.7</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="D3" t="n">
-        <v>87.2</v>
+        <v>88.8</v>
       </c>
       <c r="E3" t="n">
-        <v>0.252</v>
+        <v>0.219</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6104000000000001</v>
+        <v>0.6081</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0102</v>
+        <v>0.024</v>
       </c>
       <c r="H3" t="n">
-        <v>85.90000000000001</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>1.2</v>
+        <v>0.2</v>
       </c>
       <c r="J3" t="n">
-        <v>12.9</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="4">
@@ -1704,31 +1704,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9.9</v>
+        <v>10.1</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="D4" t="n">
-        <v>89.8</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>0.201</v>
+        <v>0.207</v>
       </c>
       <c r="F4" t="n">
-        <v>0.496</v>
+        <v>0.5278</v>
       </c>
       <c r="G4" t="n">
-        <v>0.013</v>
+        <v>0.022</v>
       </c>
       <c r="H4" t="n">
-        <v>96.90000000000001</v>
+        <v>99.8</v>
       </c>
       <c r="I4" t="n">
-        <v>1.4</v>
+        <v>0.1</v>
       </c>
       <c r="J4" t="n">
-        <v>1.7</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="5">
@@ -1738,31 +1738,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10.4</v>
+        <v>4.7</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>89.2</v>
+        <v>95.3</v>
       </c>
       <c r="E5" t="n">
-        <v>0.212</v>
+        <v>0.094</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7204</v>
+        <v>0.6698</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0178</v>
+        <v>0.0011</v>
       </c>
       <c r="H5" t="n">
-        <v>22.2</v>
+        <v>77.3</v>
       </c>
       <c r="I5" t="n">
-        <v>75</v>
+        <v>21.9</v>
       </c>
       <c r="J5" t="n">
-        <v>2.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="6">
@@ -1772,31 +1772,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6.4</v>
+        <v>2.4</v>
       </c>
       <c r="C6" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="D6" t="n">
-        <v>93</v>
+        <v>97.3</v>
       </c>
       <c r="E6" t="n">
-        <v>0.134</v>
+        <v>0.051</v>
       </c>
       <c r="F6" t="n">
-        <v>0.3679</v>
+        <v>0.1316</v>
       </c>
       <c r="G6" t="n">
-        <v>0.048</v>
+        <v>0.059</v>
       </c>
       <c r="H6" t="n">
-        <v>27.5</v>
+        <v>80.2</v>
       </c>
       <c r="I6" t="n">
-        <v>70.5</v>
+        <v>18.9</v>
       </c>
       <c r="J6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1868,28 +1868,28 @@
         <v>5.5</v>
       </c>
       <c r="C12" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="D12" t="n">
-        <v>94.3</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="E12" t="n">
-        <v>0.112</v>
+        <v>0.114</v>
       </c>
       <c r="F12" t="n">
-        <v>0.3201</v>
+        <v>0.2342</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0205</v>
+        <v>0.0315</v>
       </c>
       <c r="H12" t="n">
-        <v>76.09999999999999</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>1.6</v>
+        <v>0.4</v>
       </c>
       <c r="J12" t="n">
-        <v>22.4</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="13">
@@ -1899,31 +1899,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3.8</v>
+        <v>5.2</v>
       </c>
       <c r="C13" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D13" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.284</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.0527</v>
+      </c>
+      <c r="H13" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="J13" t="n">
         <v>0.1</v>
-      </c>
-      <c r="D13" t="n">
-        <v>96.2</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.076</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0.2461</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.0066</v>
-      </c>
-      <c r="H13" t="n">
-        <v>96.40000000000001</v>
-      </c>
-      <c r="I13" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="J13" t="n">
-        <v>1.1</v>
       </c>
     </row>
     <row r="14">
@@ -1933,31 +1933,31 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6.7</v>
+        <v>2.9</v>
       </c>
       <c r="C14" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D14" t="n">
-        <v>93.2</v>
+        <v>96.7</v>
       </c>
       <c r="E14" t="n">
-        <v>0.135</v>
+        <v>0.061</v>
       </c>
       <c r="F14" t="n">
-        <v>0.512</v>
+        <v>0.5587</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0092</v>
+        <v>0.0598</v>
       </c>
       <c r="H14" t="n">
-        <v>22.3</v>
+        <v>77.7</v>
       </c>
       <c r="I14" t="n">
-        <v>76.09999999999999</v>
+        <v>21.6</v>
       </c>
       <c r="J14" t="n">
-        <v>1.6</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="15">
@@ -1967,31 +1967,31 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4.3</v>
+        <v>1.3</v>
       </c>
       <c r="C15" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="D15" t="n">
-        <v>95.5</v>
+        <v>98.3</v>
       </c>
       <c r="E15" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.03</v>
       </c>
       <c r="F15" t="n">
-        <v>0.1273</v>
+        <v>0.5318000000000001</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0179</v>
+        <v>0.1269</v>
       </c>
       <c r="H15" t="n">
-        <v>27.9</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="I15" t="n">
-        <v>70.3</v>
+        <v>14.6</v>
       </c>
       <c r="J15" t="n">
-        <v>1.8</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="19">
@@ -2060,31 +2060,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>5</v>
+        <v>5.6</v>
       </c>
       <c r="C21" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>94.09999999999999</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="E21" t="n">
-        <v>0.109</v>
+        <v>0.122</v>
       </c>
       <c r="F21" t="n">
-        <v>0.4244</v>
+        <v>0.5897</v>
       </c>
       <c r="G21" t="n">
-        <v>0.07679999999999999</v>
+        <v>0.0805</v>
       </c>
       <c r="H21" t="n">
-        <v>80.3</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>1.7</v>
+        <v>0.5</v>
       </c>
       <c r="J21" t="n">
-        <v>18</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="22">
@@ -2094,31 +2094,31 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3.6</v>
+        <v>5.3</v>
       </c>
       <c r="C22" t="n">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
       <c r="D22" t="n">
-        <v>95.59999999999999</v>
+        <v>93.3</v>
       </c>
       <c r="E22" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="F22" t="n">
-        <v>0.5947</v>
+        <v>0.3716</v>
       </c>
       <c r="G22" t="n">
-        <v>0.09719999999999999</v>
+        <v>0.1129</v>
       </c>
       <c r="H22" t="n">
-        <v>97.59999999999999</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="I22" t="n">
-        <v>1.7</v>
+        <v>0.2</v>
       </c>
       <c r="J22" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="23">
@@ -2128,31 +2128,31 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>5.6</v>
+        <v>2.1</v>
       </c>
       <c r="C23" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>93.3</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="E23" t="n">
-        <v>0.122</v>
+        <v>0.052</v>
       </c>
       <c r="F23" t="n">
-        <v>0.4766</v>
+        <v>0.4555</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0896</v>
+        <v>0.1857</v>
       </c>
       <c r="H23" t="n">
-        <v>28.7</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="I23" t="n">
-        <v>69.40000000000001</v>
+        <v>18.6</v>
       </c>
       <c r="J23" t="n">
-        <v>1.9</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="24">
@@ -2162,31 +2162,31 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3.5</v>
+        <v>0.9</v>
       </c>
       <c r="C24" t="n">
         <v>0.6</v>
       </c>
       <c r="D24" t="n">
-        <v>95.90000000000001</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="E24" t="n">
-        <v>0.076</v>
+        <v>0.025</v>
       </c>
       <c r="F24" t="n">
-        <v>0.4585</v>
+        <v>1.8756</v>
       </c>
       <c r="G24" t="n">
-        <v>0.0755</v>
+        <v>0.2482</v>
       </c>
       <c r="H24" t="n">
-        <v>36.8</v>
+        <v>81.8</v>
       </c>
       <c r="I24" t="n">
-        <v>62.3</v>
+        <v>17.2</v>
       </c>
       <c r="J24" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="28">
@@ -2255,31 +2255,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>5.7</v>
+        <v>6.1</v>
       </c>
       <c r="C30" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="D30" t="n">
-        <v>94.09999999999999</v>
+        <v>93.8</v>
       </c>
       <c r="E30" t="n">
-        <v>0.116</v>
+        <v>0.122</v>
       </c>
       <c r="F30" t="n">
-        <v>0.6096</v>
+        <v>0.5649</v>
       </c>
       <c r="G30" t="n">
-        <v>0.021</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="H30" t="n">
-        <v>71.09999999999999</v>
+        <v>98.7</v>
       </c>
       <c r="I30" t="n">
-        <v>1.9</v>
+        <v>0.5</v>
       </c>
       <c r="J30" t="n">
-        <v>27</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="31">
@@ -2289,31 +2289,31 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3.4</v>
+        <v>5.8</v>
       </c>
       <c r="C31" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="D31" t="n">
-        <v>96.3</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="E31" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.117</v>
       </c>
       <c r="F31" t="n">
-        <v>0.9801</v>
+        <v>0.5338000000000001</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0482</v>
+        <v>0.0131</v>
       </c>
       <c r="H31" t="n">
-        <v>94.59999999999999</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="I31" t="n">
-        <v>3.4</v>
+        <v>0.2</v>
       </c>
       <c r="J31" t="n">
-        <v>2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="32">
@@ -2323,31 +2323,31 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>6.8</v>
+        <v>3.1</v>
       </c>
       <c r="C32" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="D32" t="n">
-        <v>92.8</v>
+        <v>96.7</v>
       </c>
       <c r="E32" t="n">
-        <v>0.14</v>
+        <v>0.065</v>
       </c>
       <c r="F32" t="n">
-        <v>0.4947</v>
+        <v>0.5235</v>
       </c>
       <c r="G32" t="n">
-        <v>0.0253</v>
+        <v>0.0341</v>
       </c>
       <c r="H32" t="n">
-        <v>24.2</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="I32" t="n">
-        <v>72.7</v>
+        <v>22.6</v>
       </c>
       <c r="J32" t="n">
-        <v>3.1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="33">
@@ -2357,31 +2357,31 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4.4</v>
+        <v>1.7</v>
       </c>
       <c r="C33" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D33" t="n">
-        <v>95.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="E33" t="n">
-        <v>0.094</v>
+        <v>0.034</v>
       </c>
       <c r="F33" t="n">
-        <v>0.3522</v>
+        <v>0.6516</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0531</v>
+        <v>0.0409</v>
       </c>
       <c r="H33" t="n">
-        <v>29</v>
+        <v>78.7</v>
       </c>
       <c r="I33" t="n">
-        <v>68.5</v>
+        <v>20.4</v>
       </c>
       <c r="J33" t="n">
-        <v>2.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="37">
@@ -2450,31 +2450,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>8.300000000000001</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="C39" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="D39" t="n">
-        <v>91.2</v>
+        <v>90.3</v>
       </c>
       <c r="E39" t="n">
-        <v>0.172</v>
+        <v>0.178</v>
       </c>
       <c r="F39" t="n">
-        <v>0.5383</v>
+        <v>0.4574</v>
       </c>
       <c r="G39" t="n">
-        <v>0.0269</v>
+        <v>0.08169999999999999</v>
       </c>
       <c r="H39" t="n">
-        <v>61.2</v>
+        <v>98.2</v>
       </c>
       <c r="I39" t="n">
-        <v>2.1</v>
+        <v>0.9</v>
       </c>
       <c r="J39" t="n">
-        <v>36.7</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="40">
@@ -2484,31 +2484,31 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>4.6</v>
+        <v>7.6</v>
       </c>
       <c r="C40" t="n">
-        <v>0.1</v>
+        <v>1.1</v>
       </c>
       <c r="D40" t="n">
-        <v>95.3</v>
+        <v>91.2</v>
       </c>
       <c r="E40" t="n">
-        <v>0.093</v>
+        <v>0.164</v>
       </c>
       <c r="F40" t="n">
-        <v>0.5639999999999999</v>
+        <v>0.4937</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0065</v>
+        <v>0.0697</v>
       </c>
       <c r="H40" t="n">
-        <v>94.3</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="I40" t="n">
-        <v>3.2</v>
+        <v>0.8</v>
       </c>
       <c r="J40" t="n">
-        <v>2.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="41">
@@ -2518,31 +2518,31 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>12.7</v>
+        <v>5.5</v>
       </c>
       <c r="C41" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="D41" t="n">
-        <v>87.09999999999999</v>
+        <v>94</v>
       </c>
       <c r="E41" t="n">
-        <v>0.257</v>
+        <v>0.115</v>
       </c>
       <c r="F41" t="n">
-        <v>0.5324</v>
+        <v>0.4356</v>
       </c>
       <c r="G41" t="n">
-        <v>0.0083</v>
+        <v>0.0465</v>
       </c>
       <c r="H41" t="n">
-        <v>20.2</v>
+        <v>74.5</v>
       </c>
       <c r="I41" t="n">
-        <v>77.09999999999999</v>
+        <v>24.8</v>
       </c>
       <c r="J41" t="n">
-        <v>2.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="42">
@@ -2552,31 +2552,31 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>8.4</v>
+        <v>2.5</v>
       </c>
       <c r="C42" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>91.09999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="E42" t="n">
-        <v>0.173</v>
+        <v>0.059</v>
       </c>
       <c r="F42" t="n">
-        <v>0.3491</v>
+        <v>0.4346</v>
       </c>
       <c r="G42" t="n">
-        <v>0.0258</v>
+        <v>0.172</v>
       </c>
       <c r="H42" t="n">
-        <v>24</v>
+        <v>80.8</v>
       </c>
       <c r="I42" t="n">
-        <v>74</v>
+        <v>18.9</v>
       </c>
       <c r="J42" t="n">
-        <v>2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="46">
@@ -2645,31 +2645,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="C48" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="D48" t="n">
-        <v>92.2</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="E48" t="n">
-        <v>0.152</v>
+        <v>0.151</v>
       </c>
       <c r="F48" t="n">
-        <v>0.5006</v>
+        <v>0.4909</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0311</v>
+        <v>0.0452</v>
       </c>
       <c r="H48" t="n">
-        <v>75.59999999999999</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="I48" t="n">
-        <v>1.7</v>
+        <v>0.5</v>
       </c>
       <c r="J48" t="n">
-        <v>22.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="49">
@@ -2679,31 +2679,31 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>5.1</v>
+        <v>6.8</v>
       </c>
       <c r="C49" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D49" t="n">
+        <v>92.5</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.4422</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.0541</v>
+      </c>
+      <c r="H49" t="n">
+        <v>99.5</v>
+      </c>
+      <c r="I49" t="n">
         <v>0.3</v>
       </c>
-      <c r="D49" t="n">
-        <v>94.7</v>
-      </c>
-      <c r="E49" t="n">
-        <v>0.104</v>
-      </c>
-      <c r="F49" t="n">
-        <v>0.5762</v>
-      </c>
-      <c r="G49" t="n">
-        <v>0.0343</v>
-      </c>
-      <c r="H49" t="n">
-        <v>96.09999999999999</v>
-      </c>
-      <c r="I49" t="n">
-        <v>2.3</v>
-      </c>
       <c r="J49" t="n">
-        <v>1.6</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="50">
@@ -2713,31 +2713,31 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>8.4</v>
+        <v>3.7</v>
       </c>
       <c r="C50" t="n">
         <v>0.4</v>
       </c>
       <c r="D50" t="n">
-        <v>91.09999999999999</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="E50" t="n">
-        <v>0.173</v>
+        <v>0.077</v>
       </c>
       <c r="F50" t="n">
-        <v>0.5472</v>
+        <v>0.5286</v>
       </c>
       <c r="G50" t="n">
-        <v>0.03</v>
+        <v>0.0654</v>
       </c>
       <c r="H50" t="n">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="I50" t="n">
-        <v>74.5</v>
+        <v>22.3</v>
       </c>
       <c r="J50" t="n">
-        <v>2.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="51">
@@ -2747,31 +2747,31 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>5.4</v>
+        <v>1.8</v>
       </c>
       <c r="C51" t="n">
         <v>0.5</v>
       </c>
       <c r="D51" t="n">
-        <v>94.09999999999999</v>
+        <v>97.8</v>
       </c>
       <c r="E51" t="n">
-        <v>0.113</v>
+        <v>0.04</v>
       </c>
       <c r="F51" t="n">
-        <v>0.331</v>
+        <v>0.725</v>
       </c>
       <c r="G51" t="n">
-        <v>0.0441</v>
+        <v>0.1294</v>
       </c>
       <c r="H51" t="n">
-        <v>28.2</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="I51" t="n">
-        <v>69.90000000000001</v>
+        <v>18.2</v>
       </c>
       <c r="J51" t="n">
-        <v>1.9</v>
+        <v>0.7</v>
       </c>
     </row>
   </sheetData>
@@ -2854,31 +2854,31 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D3" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.0134</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.0492</v>
+      </c>
+      <c r="H3" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="I3" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="J3" t="n">
         <v>0.3</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
-        <v>99.7</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-0.0361</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.0256</v>
-      </c>
-      <c r="H3" t="n">
-        <v>14.1</v>
-      </c>
-      <c r="I3" t="n">
-        <v>35.9</v>
-      </c>
-      <c r="J3" t="n">
-        <v>50</v>
       </c>
     </row>
     <row r="4">
@@ -2888,31 +2888,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>7.7</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D4" t="n">
-        <v>100</v>
+        <v>92.2</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>0.154</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>0.0111</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>0.0043</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>36.8</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>62.8</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="5">
@@ -2922,31 +2922,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>42.3</v>
+        <v>16.3</v>
       </c>
       <c r="C5" t="n">
-        <v>13.9</v>
+        <v>2.3</v>
       </c>
       <c r="D5" t="n">
-        <v>43.8</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="E5" t="n">
-        <v>0.984</v>
+        <v>0.348</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0114</v>
+        <v>0.0112</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1411</v>
+        <v>0.0658</v>
       </c>
       <c r="H5" t="n">
-        <v>3.9</v>
+        <v>23.9</v>
       </c>
       <c r="I5" t="n">
-        <v>95.5</v>
+        <v>75.8</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="6">
@@ -2956,28 +2956,28 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7.4</v>
+        <v>6.5</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="D6" t="n">
-        <v>92.3</v>
+        <v>93</v>
       </c>
       <c r="E6" t="n">
-        <v>0.151</v>
+        <v>0.135</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.0056</v>
+        <v>0.0022</v>
       </c>
       <c r="G6" t="n">
-        <v>0.021</v>
+        <v>0.0382</v>
       </c>
       <c r="H6" t="n">
-        <v>25.5</v>
+        <v>29.8</v>
       </c>
       <c r="I6" t="n">
-        <v>73.90000000000001</v>
+        <v>69.5</v>
       </c>
       <c r="J6" t="n">
         <v>0.7</v>
@@ -3049,31 +3049,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.1</v>
+        <v>7.9</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="D12" t="n">
-        <v>99.90000000000001</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>0.002</v>
+        <v>0.185</v>
       </c>
       <c r="F12" t="n">
-        <v>0.082</v>
+        <v>-0.0476</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0476</v>
+        <v>0.148</v>
       </c>
       <c r="H12" t="n">
-        <v>14.3</v>
+        <v>24.1</v>
       </c>
       <c r="I12" t="n">
-        <v>76.2</v>
+        <v>75.7</v>
       </c>
       <c r="J12" t="n">
-        <v>9.5</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="13">
@@ -3083,31 +3083,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D13" t="n">
-        <v>100</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>0.063</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>-0.0377</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>0.08069999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>58.7</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="14">
@@ -3117,31 +3117,31 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>20</v>
+        <v>7.5</v>
       </c>
       <c r="C14" t="n">
-        <v>6.5</v>
+        <v>2.9</v>
       </c>
       <c r="D14" t="n">
-        <v>73.5</v>
+        <v>89.5</v>
       </c>
       <c r="E14" t="n">
-        <v>0.466</v>
+        <v>0.18</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.0163</v>
+        <v>-0.0432</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1402</v>
+        <v>0.1624</v>
       </c>
       <c r="H14" t="n">
-        <v>3.7</v>
+        <v>23.4</v>
       </c>
       <c r="I14" t="n">
-        <v>96.09999999999999</v>
+        <v>76.5</v>
       </c>
       <c r="J14" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="15">
@@ -3151,31 +3151,31 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="C15" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="D15" t="n">
-        <v>97.40000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="E15" t="n">
-        <v>0.051</v>
+        <v>0.059</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.0708</v>
+        <v>-0.0375</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0132</v>
+        <v>0.0563</v>
       </c>
       <c r="H15" t="n">
-        <v>35.2</v>
+        <v>37.9</v>
       </c>
       <c r="I15" t="n">
-        <v>64.8</v>
+        <v>61.9</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="19">
@@ -3244,31 +3244,31 @@
         </is>
       </c>
       <c r="B21" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>89.7</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.204</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-0.0149</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.0097</v>
+      </c>
+      <c r="H21" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="I21" t="n">
+        <v>69.3</v>
+      </c>
+      <c r="J21" t="n">
         <v>0.1</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" t="n">
-        <v>99.90000000000001</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0.0847</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.0588</v>
-      </c>
-      <c r="H21" t="n">
-        <v>11.8</v>
-      </c>
-      <c r="I21" t="n">
-        <v>41.2</v>
-      </c>
-      <c r="J21" t="n">
-        <v>47.1</v>
       </c>
     </row>
     <row r="22">
@@ -3278,28 +3278,28 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0</v>
+        <v>3.9</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>100</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>0.078</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>-0.0186</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>0.0026</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -3312,28 +3312,28 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>20.2</v>
+        <v>9.5</v>
       </c>
       <c r="C23" t="n">
-        <v>8.800000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="D23" t="n">
-        <v>71</v>
+        <v>89.8</v>
       </c>
       <c r="E23" t="n">
-        <v>0.492</v>
+        <v>0.197</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0003</v>
+        <v>-0.0073</v>
       </c>
       <c r="G23" t="n">
-        <v>0.1795</v>
+        <v>0.0329</v>
       </c>
       <c r="H23" t="n">
-        <v>4.6</v>
+        <v>28.7</v>
       </c>
       <c r="I23" t="n">
-        <v>95.40000000000001</v>
+        <v>71.2</v>
       </c>
       <c r="J23" t="n">
         <v>0.1</v>
@@ -3346,7 +3346,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="C24" t="n">
         <v>0.4</v>
@@ -3355,22 +3355,22 @@
         <v>96.3</v>
       </c>
       <c r="E24" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0027</v>
+        <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0.0556</v>
+        <v>0.0612</v>
       </c>
       <c r="H24" t="n">
-        <v>38.2</v>
+        <v>37.3</v>
       </c>
       <c r="I24" t="n">
-        <v>61.6</v>
+        <v>62.7</v>
       </c>
       <c r="J24" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -3439,31 +3439,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D30" t="n">
-        <v>100</v>
+        <v>90.2</v>
       </c>
       <c r="E30" t="n">
-        <v>0.001</v>
+        <v>0.195</v>
       </c>
       <c r="F30" t="n">
-        <v>0.0433</v>
+        <v>0.0259</v>
       </c>
       <c r="G30" t="n">
-        <v>0.2</v>
+        <v>0.0031</v>
       </c>
       <c r="H30" t="n">
-        <v>30</v>
+        <v>28.5</v>
       </c>
       <c r="I30" t="n">
-        <v>30</v>
+        <v>71.2</v>
       </c>
       <c r="J30" t="n">
-        <v>40</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="31">
@@ -3473,28 +3473,28 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0</v>
+        <v>3.1</v>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="D31" t="n">
-        <v>100</v>
+        <v>96.3</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>0.0128</v>
       </c>
       <c r="G31" t="n">
-        <v>0</v>
+        <v>0.0859</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -3507,31 +3507,31 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>20.5</v>
+        <v>9.5</v>
       </c>
       <c r="C32" t="n">
-        <v>7.3</v>
+        <v>0.2</v>
       </c>
       <c r="D32" t="n">
-        <v>72.2</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="E32" t="n">
-        <v>0.482</v>
+        <v>0.191</v>
       </c>
       <c r="F32" t="n">
-        <v>0.0279</v>
+        <v>0.0235</v>
       </c>
       <c r="G32" t="n">
-        <v>0.151</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="H32" t="n">
-        <v>4.4</v>
+        <v>26.4</v>
       </c>
       <c r="I32" t="n">
-        <v>95.5</v>
+        <v>73.3</v>
       </c>
       <c r="J32" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="33">
@@ -3541,28 +3541,28 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="C33" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D33" t="n">
-        <v>97.2</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="E33" t="n">
-        <v>0.055</v>
+        <v>0.065</v>
       </c>
       <c r="F33" t="n">
-        <v>0.0126</v>
+        <v>0.0122</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0124</v>
+        <v>0.0567</v>
       </c>
       <c r="H33" t="n">
-        <v>40.9</v>
+        <v>32.3</v>
       </c>
       <c r="I33" t="n">
-        <v>59.1</v>
+        <v>67.7</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -3634,31 +3634,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.1</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="C39" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="D39" t="n">
+        <v>86.59999999999999</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.221</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.0336</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.2133</v>
+      </c>
+      <c r="H39" t="n">
+        <v>20</v>
+      </c>
+      <c r="I39" t="n">
+        <v>80</v>
+      </c>
+      <c r="J39" t="n">
         <v>0</v>
-      </c>
-      <c r="D39" t="n">
-        <v>99.90000000000001</v>
-      </c>
-      <c r="E39" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="F39" t="n">
-        <v>0.0603</v>
-      </c>
-      <c r="G39" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="H39" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="I39" t="n">
-        <v>31.2</v>
-      </c>
-      <c r="J39" t="n">
-        <v>56.2</v>
       </c>
     </row>
     <row r="40">
@@ -3668,28 +3668,28 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="D40" t="n">
-        <v>100</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="E40" t="n">
-        <v>0</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>0.0277</v>
       </c>
       <c r="G40" t="n">
-        <v>0</v>
+        <v>0.1288</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>38.6</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>61.4</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -3702,28 +3702,28 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>19.4</v>
+        <v>8.4</v>
       </c>
       <c r="C41" t="n">
-        <v>16.4</v>
+        <v>4.7</v>
       </c>
       <c r="D41" t="n">
-        <v>64.2</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="E41" t="n">
-        <v>0.552</v>
+        <v>0.215</v>
       </c>
       <c r="F41" t="n">
-        <v>0.0261</v>
+        <v>0.0341</v>
       </c>
       <c r="G41" t="n">
-        <v>0.2978</v>
+        <v>0.2191</v>
       </c>
       <c r="H41" t="n">
-        <v>3</v>
+        <v>18.5</v>
       </c>
       <c r="I41" t="n">
-        <v>96.90000000000001</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="J41" t="n">
         <v>0.1</v>
@@ -3736,31 +3736,31 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="C42" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="D42" t="n">
-        <v>97.7</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="E42" t="n">
-        <v>0.043</v>
+        <v>0.064</v>
       </c>
       <c r="F42" t="n">
-        <v>0.0264</v>
+        <v>0.0328</v>
       </c>
       <c r="G42" t="n">
-        <v>0.0684</v>
+        <v>0.1238</v>
       </c>
       <c r="H42" t="n">
-        <v>34.7</v>
+        <v>36.4</v>
       </c>
       <c r="I42" t="n">
-        <v>64.90000000000001</v>
+        <v>63.6</v>
       </c>
       <c r="J42" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -3829,31 +3829,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>0.1</v>
+        <v>10.8</v>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="D48" t="n">
-        <v>99.90000000000001</v>
+        <v>87.3</v>
       </c>
       <c r="E48" t="n">
-        <v>0.003</v>
+        <v>0.235</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0469</v>
+        <v>0.0021</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0914</v>
+        <v>0.08459999999999999</v>
       </c>
       <c r="H48" t="n">
-        <v>14.8</v>
+        <v>26.2</v>
       </c>
       <c r="I48" t="n">
-        <v>41.5</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="J48" t="n">
-        <v>43.7</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="49">
@@ -3863,31 +3863,31 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0</v>
+        <v>4.1</v>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D49" t="n">
-        <v>100</v>
+        <v>95.5</v>
       </c>
       <c r="E49" t="n">
-        <v>0</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="F49" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="G49" t="n">
-        <v>0</v>
+        <v>0.0605</v>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>38.6</v>
       </c>
       <c r="I49" t="n">
-        <v>0</v>
+        <v>61.2</v>
       </c>
       <c r="J49" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="50">
@@ -3897,31 +3897,31 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>24.5</v>
+        <v>10.2</v>
       </c>
       <c r="C50" t="n">
-        <v>10.6</v>
+        <v>2.1</v>
       </c>
       <c r="D50" t="n">
-        <v>64.90000000000001</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="E50" t="n">
-        <v>0.595</v>
+        <v>0.226</v>
       </c>
       <c r="F50" t="n">
-        <v>0.009900000000000001</v>
+        <v>0.0037</v>
       </c>
       <c r="G50" t="n">
-        <v>0.1819</v>
+        <v>0.0978</v>
       </c>
       <c r="H50" t="n">
-        <v>3.9</v>
+        <v>24.1</v>
       </c>
       <c r="I50" t="n">
-        <v>95.8</v>
+        <v>75.7</v>
       </c>
       <c r="J50" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="51">
@@ -3931,28 +3931,28 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="C51" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="D51" t="n">
-        <v>96.2</v>
+        <v>95.8</v>
       </c>
       <c r="E51" t="n">
-        <v>0.074</v>
+        <v>0.078</v>
       </c>
       <c r="F51" t="n">
-        <v>-0.0069</v>
+        <v>0.002</v>
       </c>
       <c r="G51" t="n">
-        <v>0.0341</v>
+        <v>0.0672</v>
       </c>
       <c r="H51" t="n">
-        <v>32.9</v>
+        <v>34</v>
       </c>
       <c r="I51" t="n">
-        <v>66.8</v>
+        <v>65.8</v>
       </c>
       <c r="J51" t="n">
         <v>0.3</v>
@@ -4038,31 +4038,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.1</v>
+        <v>7.8</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D3" t="n">
-        <v>98.8</v>
+        <v>91.8</v>
       </c>
       <c r="E3" t="n">
-        <v>0.023</v>
+        <v>0.16</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0682</v>
+        <v>0.0256</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0315</v>
+        <v>0.0219</v>
       </c>
       <c r="H3" t="n">
-        <v>56.7</v>
+        <v>68.8</v>
       </c>
       <c r="I3" t="n">
-        <v>11.8</v>
+        <v>30.2</v>
       </c>
       <c r="J3" t="n">
-        <v>31.5</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="4">
@@ -4072,31 +4072,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1</v>
+        <v>5.1</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D4" t="n">
-        <v>99.8</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>0.004</v>
+        <v>0.105</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0785</v>
+        <v>0.0091</v>
       </c>
       <c r="G4" t="n">
-        <v>0.15</v>
+        <v>0.0359</v>
       </c>
       <c r="H4" t="n">
-        <v>50</v>
+        <v>78.2</v>
       </c>
       <c r="I4" t="n">
-        <v>47.5</v>
+        <v>21.3</v>
       </c>
       <c r="J4" t="n">
-        <v>2.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="5">
@@ -4106,31 +4106,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8.6</v>
+        <v>5.9</v>
       </c>
       <c r="C5" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="D5" t="n">
-        <v>90.7</v>
+        <v>93.8</v>
       </c>
       <c r="E5" t="n">
-        <v>0.179</v>
+        <v>0.121</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0192</v>
+        <v>0.0182</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0368</v>
+        <v>0.0321</v>
       </c>
       <c r="H5" t="n">
-        <v>41.7</v>
+        <v>51.1</v>
       </c>
       <c r="I5" t="n">
-        <v>56.8</v>
+        <v>47.8</v>
       </c>
       <c r="J5" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="6">
@@ -4140,31 +4140,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>1.9</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>95</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="E6" t="n">
-        <v>0.09</v>
+        <v>0.048</v>
       </c>
       <c r="F6" t="n">
-        <v>0.024</v>
+        <v>0.0232</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1061</v>
+        <v>0.204</v>
       </c>
       <c r="H6" t="n">
-        <v>46.2</v>
+        <v>51.2</v>
       </c>
       <c r="I6" t="n">
-        <v>52.5</v>
+        <v>48</v>
       </c>
       <c r="J6" t="n">
-        <v>1.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="10">
@@ -4233,31 +4233,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.6</v>
+        <v>5.7</v>
       </c>
       <c r="C12" t="n">
-        <v>0.1</v>
+        <v>1.4</v>
       </c>
       <c r="D12" t="n">
-        <v>99.40000000000001</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>0.012</v>
+        <v>0.127</v>
       </c>
       <c r="F12" t="n">
-        <v>0.068</v>
+        <v>0.0135</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0448</v>
+        <v>0.1096</v>
       </c>
       <c r="H12" t="n">
-        <v>50</v>
+        <v>64.3</v>
       </c>
       <c r="I12" t="n">
-        <v>17.2</v>
+        <v>35</v>
       </c>
       <c r="J12" t="n">
-        <v>32.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="13">
@@ -4267,31 +4267,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1</v>
+        <v>3.8</v>
       </c>
       <c r="C13" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="D13" t="n">
-        <v>99.8</v>
+        <v>95.7</v>
       </c>
       <c r="E13" t="n">
-        <v>0.004</v>
+        <v>0.081</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1955</v>
+        <v>-0</v>
       </c>
       <c r="G13" t="n">
-        <v>0.2</v>
+        <v>0.0677</v>
       </c>
       <c r="H13" t="n">
-        <v>80</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>12.5</v>
+        <v>24.4</v>
       </c>
       <c r="J13" t="n">
-        <v>7.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="14">
@@ -4301,31 +4301,31 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>7.1</v>
+        <v>4.5</v>
       </c>
       <c r="C14" t="n">
-        <v>2.3</v>
+        <v>0.7</v>
       </c>
       <c r="D14" t="n">
-        <v>90.59999999999999</v>
+        <v>94.8</v>
       </c>
       <c r="E14" t="n">
-        <v>0.165</v>
+        <v>0.096</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0244</v>
+        <v>0.0141</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1419</v>
+        <v>0.0756</v>
       </c>
       <c r="H14" t="n">
-        <v>36</v>
+        <v>44.4</v>
       </c>
       <c r="I14" t="n">
-        <v>62.6</v>
+        <v>54.7</v>
       </c>
       <c r="J14" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -4335,31 +4335,31 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3.2</v>
+        <v>1.7</v>
       </c>
       <c r="C15" t="n">
-        <v>1.1</v>
+        <v>0.6</v>
       </c>
       <c r="D15" t="n">
-        <v>95.7</v>
+        <v>97.7</v>
       </c>
       <c r="E15" t="n">
-        <v>0.074</v>
+        <v>0.04</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0416</v>
+        <v>0.035</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1425</v>
+        <v>0.1496</v>
       </c>
       <c r="H15" t="n">
-        <v>39</v>
+        <v>44.2</v>
       </c>
       <c r="I15" t="n">
-        <v>60.3</v>
+        <v>54.6</v>
       </c>
       <c r="J15" t="n">
-        <v>0.7</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="19">
@@ -4428,31 +4428,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1.6</v>
+        <v>6.7</v>
       </c>
       <c r="C21" t="n">
-        <v>0.4</v>
+        <v>1.3</v>
       </c>
       <c r="D21" t="n">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E21" t="n">
-        <v>0.036</v>
+        <v>0.147</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0234</v>
+        <v>0.0024</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0979</v>
+        <v>0.0878</v>
       </c>
       <c r="H21" t="n">
-        <v>54.4</v>
+        <v>73.2</v>
       </c>
       <c r="I21" t="n">
-        <v>9.5</v>
+        <v>25.4</v>
       </c>
       <c r="J21" t="n">
-        <v>36.1</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="22">
@@ -4462,31 +4462,31 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.3</v>
+        <v>4.9</v>
       </c>
       <c r="C22" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>99.5</v>
+        <v>94.2</v>
       </c>
       <c r="E22" t="n">
-        <v>0.008</v>
+        <v>0.107</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.0236</v>
+        <v>-0.013</v>
       </c>
       <c r="G22" t="n">
-        <v>0.1957</v>
+        <v>0.0897</v>
       </c>
       <c r="H22" t="n">
-        <v>69.59999999999999</v>
+        <v>80.3</v>
       </c>
       <c r="I22" t="n">
-        <v>26.1</v>
+        <v>18.6</v>
       </c>
       <c r="J22" t="n">
-        <v>4.3</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="23">
@@ -4496,31 +4496,31 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>9.300000000000001</v>
+        <v>4.8</v>
       </c>
       <c r="C23" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="D23" t="n">
-        <v>89.3</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="E23" t="n">
-        <v>0.2</v>
+        <v>0.107</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0184</v>
+        <v>0.004</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0694</v>
+        <v>0.0998</v>
       </c>
       <c r="H23" t="n">
-        <v>43.2</v>
+        <v>48.6</v>
       </c>
       <c r="I23" t="n">
-        <v>54.8</v>
+        <v>48.8</v>
       </c>
       <c r="J23" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="24">
@@ -4530,31 +4530,31 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="C24" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D24" t="n">
-        <v>95</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="E24" t="n">
-        <v>0.094</v>
+        <v>0.046</v>
       </c>
       <c r="F24" t="n">
-        <v>0.025</v>
+        <v>-0.0295</v>
       </c>
       <c r="G24" t="n">
-        <v>0.0582</v>
+        <v>0.0267</v>
       </c>
       <c r="H24" t="n">
-        <v>43.9</v>
+        <v>46.6</v>
       </c>
       <c r="I24" t="n">
-        <v>55.1</v>
+        <v>51.3</v>
       </c>
       <c r="J24" t="n">
-        <v>1.1</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="28">
@@ -4623,31 +4623,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.7</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="C30" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="D30" t="n">
-        <v>99.09999999999999</v>
+        <v>89.7</v>
       </c>
       <c r="E30" t="n">
-        <v>0.016</v>
+        <v>0.201</v>
       </c>
       <c r="F30" t="n">
-        <v>0.1231</v>
+        <v>0.0401</v>
       </c>
       <c r="G30" t="n">
-        <v>0.1196</v>
+        <v>0.0287</v>
       </c>
       <c r="H30" t="n">
-        <v>54.9</v>
+        <v>56.2</v>
       </c>
       <c r="I30" t="n">
-        <v>13.6</v>
+        <v>43.3</v>
       </c>
       <c r="J30" t="n">
-        <v>31.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="31">
@@ -4657,31 +4657,31 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.2</v>
+        <v>3.8</v>
       </c>
       <c r="C31" t="n">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
       <c r="D31" t="n">
-        <v>99.7</v>
+        <v>95.3</v>
       </c>
       <c r="E31" t="n">
-        <v>0.005</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="F31" t="n">
-        <v>0.2072</v>
+        <v>-0.0199</v>
       </c>
       <c r="G31" t="n">
-        <v>0.3333</v>
+        <v>0.1014</v>
       </c>
       <c r="H31" t="n">
-        <v>71.90000000000001</v>
+        <v>62.1</v>
       </c>
       <c r="I31" t="n">
-        <v>26.3</v>
+        <v>37.9</v>
       </c>
       <c r="J31" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -4691,31 +4691,31 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>10.9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="C32" t="n">
-        <v>2.4</v>
+        <v>0.8</v>
       </c>
       <c r="D32" t="n">
-        <v>86.7</v>
+        <v>90.5</v>
       </c>
       <c r="E32" t="n">
-        <v>0.242</v>
+        <v>0.181</v>
       </c>
       <c r="F32" t="n">
-        <v>0.0629</v>
+        <v>0.057</v>
       </c>
       <c r="G32" t="n">
-        <v>0.0979</v>
+        <v>0.0415</v>
       </c>
       <c r="H32" t="n">
-        <v>37.5</v>
+        <v>48.7</v>
       </c>
       <c r="I32" t="n">
-        <v>61.5</v>
+        <v>50.6</v>
       </c>
       <c r="J32" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="33">
@@ -4725,31 +4725,31 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>5.2</v>
+        <v>2.3</v>
       </c>
       <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>96.7</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.057</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.0512</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.1738</v>
+      </c>
+      <c r="H33" t="n">
+        <v>45.3</v>
+      </c>
+      <c r="I33" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="J33" t="n">
         <v>0.3</v>
-      </c>
-      <c r="D33" t="n">
-        <v>94.40000000000001</v>
-      </c>
-      <c r="E33" t="n">
-        <v>0.108</v>
-      </c>
-      <c r="F33" t="n">
-        <v>0.0264</v>
-      </c>
-      <c r="G33" t="n">
-        <v>0.0302</v>
-      </c>
-      <c r="H33" t="n">
-        <v>43.7</v>
-      </c>
-      <c r="I33" t="n">
-        <v>55.1</v>
-      </c>
-      <c r="J33" t="n">
-        <v>1.2</v>
       </c>
     </row>
     <row r="37">
@@ -4818,31 +4818,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.7</v>
+        <v>5.9</v>
       </c>
       <c r="C39" t="n">
-        <v>0.1</v>
+        <v>1.4</v>
       </c>
       <c r="D39" t="n">
-        <v>99.2</v>
+        <v>92.7</v>
       </c>
       <c r="E39" t="n">
-        <v>0.015</v>
+        <v>0.133</v>
       </c>
       <c r="F39" t="n">
-        <v>-0.0171</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="G39" t="n">
-        <v>0.0539</v>
+        <v>0.1037</v>
       </c>
       <c r="H39" t="n">
-        <v>55.7</v>
+        <v>55.6</v>
       </c>
       <c r="I39" t="n">
-        <v>11.4</v>
+        <v>43.6</v>
       </c>
       <c r="J39" t="n">
-        <v>32.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="40">
@@ -4852,31 +4852,31 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.1</v>
+        <v>3.7</v>
       </c>
       <c r="C40" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="D40" t="n">
-        <v>99.59999999999999</v>
+        <v>95.8</v>
       </c>
       <c r="E40" t="n">
-        <v>0.005</v>
+        <v>0.079</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.1334</v>
+        <v>0.0114</v>
       </c>
       <c r="G40" t="n">
-        <v>0.5333</v>
+        <v>0.0675</v>
       </c>
       <c r="H40" t="n">
-        <v>73.3</v>
+        <v>68.3</v>
       </c>
       <c r="I40" t="n">
-        <v>25</v>
+        <v>30.6</v>
       </c>
       <c r="J40" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="41">
@@ -4886,31 +4886,31 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>6.2</v>
+        <v>4.8</v>
       </c>
       <c r="C41" t="n">
-        <v>1.6</v>
+        <v>1.2</v>
       </c>
       <c r="D41" t="n">
-        <v>92.2</v>
+        <v>94</v>
       </c>
       <c r="E41" t="n">
-        <v>0.14</v>
+        <v>0.108</v>
       </c>
       <c r="F41" t="n">
-        <v>-0.0057</v>
+        <v>0.0086</v>
       </c>
       <c r="G41" t="n">
-        <v>0.1147</v>
+        <v>0.107</v>
       </c>
       <c r="H41" t="n">
-        <v>34.7</v>
+        <v>38.8</v>
       </c>
       <c r="I41" t="n">
-        <v>64</v>
+        <v>60.3</v>
       </c>
       <c r="J41" t="n">
-        <v>1.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -4920,31 +4920,31 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>3.3</v>
+        <v>2.3</v>
       </c>
       <c r="C42" t="n">
-        <v>0.8</v>
+        <v>0.1</v>
       </c>
       <c r="D42" t="n">
-        <v>95.90000000000001</v>
+        <v>97.7</v>
       </c>
       <c r="E42" t="n">
-        <v>0.074</v>
+        <v>0.046</v>
       </c>
       <c r="F42" t="n">
-        <v>-0.0112</v>
+        <v>-0.0111</v>
       </c>
       <c r="G42" t="n">
-        <v>0.1031</v>
+        <v>0.0104</v>
       </c>
       <c r="H42" t="n">
-        <v>39.9</v>
+        <v>43.7</v>
       </c>
       <c r="I42" t="n">
-        <v>59.3</v>
+        <v>54.9</v>
       </c>
       <c r="J42" t="n">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="46">
@@ -5013,31 +5013,31 @@
         </is>
       </c>
       <c r="B48" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.0181</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.0703</v>
+      </c>
+      <c r="H48" t="n">
+        <v>63.5</v>
+      </c>
+      <c r="I48" t="n">
+        <v>35.7</v>
+      </c>
+      <c r="J48" t="n">
         <v>0.9</v>
-      </c>
-      <c r="C48" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D48" t="n">
-        <v>98.90000000000001</v>
-      </c>
-      <c r="E48" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="F48" t="n">
-        <v>0.0531</v>
-      </c>
-      <c r="G48" t="n">
-        <v>0.06950000000000001</v>
-      </c>
-      <c r="H48" t="n">
-        <v>54.7</v>
-      </c>
-      <c r="I48" t="n">
-        <v>11.9</v>
-      </c>
-      <c r="J48" t="n">
-        <v>33.5</v>
       </c>
     </row>
     <row r="49">
@@ -5047,31 +5047,31 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.2</v>
+        <v>4.2</v>
       </c>
       <c r="C49" t="n">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
       <c r="D49" t="n">
-        <v>99.7</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="E49" t="n">
-        <v>0.005</v>
+        <v>0.091</v>
       </c>
       <c r="F49" t="n">
-        <v>0.0648</v>
+        <v>-0.0025</v>
       </c>
       <c r="G49" t="n">
-        <v>0.2825</v>
+        <v>0.07240000000000001</v>
       </c>
       <c r="H49" t="n">
-        <v>69.59999999999999</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="I49" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J49" t="n">
-        <v>3.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="50">
@@ -5081,31 +5081,31 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>8.4</v>
+        <v>5.7</v>
       </c>
       <c r="C50" t="n">
-        <v>1.7</v>
+        <v>0.8</v>
       </c>
       <c r="D50" t="n">
-        <v>89.90000000000001</v>
+        <v>93.5</v>
       </c>
       <c r="E50" t="n">
-        <v>0.185</v>
+        <v>0.123</v>
       </c>
       <c r="F50" t="n">
-        <v>0.0238</v>
+        <v>0.0204</v>
       </c>
       <c r="G50" t="n">
-        <v>0.0921</v>
+        <v>0.0712</v>
       </c>
       <c r="H50" t="n">
-        <v>38.8</v>
+        <v>46.6</v>
       </c>
       <c r="I50" t="n">
-        <v>59.8</v>
+        <v>52.1</v>
       </c>
       <c r="J50" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="51">
@@ -5115,31 +5115,31 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>4</v>
+        <v>2.1</v>
       </c>
       <c r="C51" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="D51" t="n">
-        <v>95.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="E51" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.047</v>
       </c>
       <c r="F51" t="n">
-        <v>0.0211</v>
+        <v>0.0137</v>
       </c>
       <c r="G51" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.1129</v>
       </c>
       <c r="H51" t="n">
-        <v>42.8</v>
+        <v>46.2</v>
       </c>
       <c r="I51" t="n">
-        <v>56.2</v>
+        <v>52.6</v>
       </c>
       <c r="J51" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
   </sheetData>
@@ -5222,31 +5222,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>2.2</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="D3" t="n">
-        <v>96.8</v>
+        <v>97.5</v>
       </c>
       <c r="E3" t="n">
-        <v>0.062</v>
+        <v>0.046</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.0193</v>
+        <v>-0.0352</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0316</v>
+        <v>0.06909999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>52.5</v>
+        <v>47.8</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>33.9</v>
       </c>
       <c r="J3" t="n">
-        <v>47.5</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="4">
@@ -5256,31 +5256,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1</v>
+        <v>0.7</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="D4" t="n">
-        <v>99.90000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>0.002</v>
+        <v>0.016</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.07149999999999999</v>
+        <v>-0.0451</v>
       </c>
       <c r="G4" t="n">
-        <v>0.1538</v>
+        <v>0.116</v>
       </c>
       <c r="H4" t="n">
-        <v>100</v>
+        <v>57.5</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>40.3</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="5">
@@ -5290,31 +5290,31 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>24.1</v>
+        <v>8.4</v>
       </c>
       <c r="C5" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="D5" t="n">
-        <v>75.40000000000001</v>
+        <v>90.8</v>
       </c>
       <c r="E5" t="n">
-        <v>0.487</v>
+        <v>0.176</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0115</v>
+        <v>-0.0026</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0109</v>
+        <v>0.0441</v>
       </c>
       <c r="H5" t="n">
-        <v>18</v>
+        <v>47.6</v>
       </c>
       <c r="I5" t="n">
-        <v>81.2</v>
+        <v>52</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="6">
@@ -5324,31 +5324,31 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6.2</v>
+        <v>3.1</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="D6" t="n">
-        <v>92.8</v>
+        <v>96.7</v>
       </c>
       <c r="E6" t="n">
-        <v>0.134</v>
+        <v>0.065</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.028</v>
+        <v>-0.0473</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0736</v>
+        <v>0.0302</v>
       </c>
       <c r="H6" t="n">
-        <v>42.2</v>
+        <v>47</v>
       </c>
       <c r="I6" t="n">
-        <v>57</v>
+        <v>51.8</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="10">
@@ -5417,31 +5417,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1.3</v>
+        <v>0.6</v>
       </c>
       <c r="C12" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="D12" t="n">
-        <v>98.40000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="E12" t="n">
-        <v>0.029</v>
+        <v>0.015</v>
       </c>
       <c r="F12" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.0217</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1195</v>
+        <v>0.1786</v>
       </c>
       <c r="H12" t="n">
-        <v>48.4</v>
+        <v>41.1</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>35.7</v>
       </c>
       <c r="J12" t="n">
-        <v>51.6</v>
+        <v>23.2</v>
       </c>
     </row>
     <row r="13">
@@ -5451,31 +5451,31 @@
         </is>
       </c>
       <c r="B13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C13" t="n">
         <v>0.1</v>
       </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
       <c r="D13" t="n">
-        <v>99.90000000000001</v>
+        <v>99.8</v>
       </c>
       <c r="E13" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0212</v>
+        <v>0.0234</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0526</v>
+        <v>0.1304</v>
       </c>
       <c r="H13" t="n">
-        <v>89.5</v>
+        <v>54.3</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>43.5</v>
       </c>
       <c r="J13" t="n">
-        <v>10.5</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="14">
@@ -5485,31 +5485,31 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15.1</v>
+        <v>4.6</v>
       </c>
       <c r="C14" t="n">
-        <v>8.199999999999999</v>
+        <v>3.2</v>
       </c>
       <c r="D14" t="n">
-        <v>76.7</v>
+        <v>92.2</v>
       </c>
       <c r="E14" t="n">
-        <v>0.385</v>
+        <v>0.124</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0081</v>
+        <v>0.0231</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2131</v>
+        <v>0.2578</v>
       </c>
       <c r="H14" t="n">
-        <v>12.4</v>
+        <v>36</v>
       </c>
       <c r="I14" t="n">
-        <v>87.2</v>
+        <v>63.9</v>
       </c>
       <c r="J14" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="15">
@@ -5519,31 +5519,31 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4.2</v>
+        <v>1.1</v>
       </c>
       <c r="C15" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>97.59999999999999</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.035</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.0198</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.3668</v>
+      </c>
+      <c r="H15" t="n">
+        <v>38.8</v>
+      </c>
+      <c r="I15" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="J15" t="n">
         <v>0.3</v>
-      </c>
-      <c r="D15" t="n">
-        <v>95.5</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.08699999999999999</v>
-      </c>
-      <c r="F15" t="n">
-        <v>-0.0018</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.0319</v>
-      </c>
-      <c r="H15" t="n">
-        <v>39</v>
-      </c>
-      <c r="I15" t="n">
-        <v>60.3</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0.7</v>
       </c>
     </row>
     <row r="19">
@@ -5612,31 +5612,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1.4</v>
+        <v>0.8</v>
       </c>
       <c r="C21" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="D21" t="n">
-        <v>98.3</v>
+        <v>99</v>
       </c>
       <c r="E21" t="n">
-        <v>0.031</v>
+        <v>0.018</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0307</v>
+        <v>-0.0016</v>
       </c>
       <c r="G21" t="n">
-        <v>0.09520000000000001</v>
+        <v>0.09089999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>49.1</v>
+        <v>39.4</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>36.4</v>
       </c>
       <c r="J21" t="n">
-        <v>50.9</v>
+        <v>24.2</v>
       </c>
     </row>
     <row r="22">
@@ -5646,28 +5646,28 @@
         </is>
       </c>
       <c r="B22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C22" t="n">
         <v>0.1</v>
       </c>
-      <c r="C22" t="n">
-        <v>0</v>
-      </c>
       <c r="D22" t="n">
-        <v>99.90000000000001</v>
+        <v>99.7</v>
       </c>
       <c r="E22" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
       <c r="F22" t="n">
-        <v>0.1088</v>
+        <v>-0.0133</v>
       </c>
       <c r="G22" t="n">
-        <v>0</v>
+        <v>0.3091</v>
       </c>
       <c r="H22" t="n">
-        <v>100</v>
+        <v>58.2</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>41.8</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -5680,31 +5680,31 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>16.3</v>
+        <v>4.9</v>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
+        <v>1.1</v>
       </c>
       <c r="D23" t="n">
-        <v>81.8</v>
+        <v>94</v>
       </c>
       <c r="E23" t="n">
-        <v>0.345</v>
+        <v>0.11</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0324</v>
+        <v>0.0201</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0574</v>
+        <v>0.1022</v>
       </c>
       <c r="H23" t="n">
-        <v>14.4</v>
+        <v>41.9</v>
       </c>
       <c r="I23" t="n">
-        <v>85</v>
+        <v>57.8</v>
       </c>
       <c r="J23" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="24">
@@ -5714,28 +5714,28 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3.5</v>
+        <v>1.6</v>
       </c>
       <c r="C24" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="D24" t="n">
-        <v>96</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="E24" t="n">
-        <v>0.075</v>
+        <v>0.037</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0306</v>
+        <v>0.0435</v>
       </c>
       <c r="G24" t="n">
-        <v>0.059</v>
+        <v>0.145</v>
       </c>
       <c r="H24" t="n">
-        <v>45.8</v>
+        <v>43.3</v>
       </c>
       <c r="I24" t="n">
-        <v>53.9</v>
+        <v>56.5</v>
       </c>
       <c r="J24" t="n">
         <v>0.3</v>
@@ -5807,31 +5807,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1.2</v>
+        <v>0.9</v>
       </c>
       <c r="C30" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>98.5</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="E30" t="n">
-        <v>0.027</v>
+        <v>0.018</v>
       </c>
       <c r="F30" t="n">
-        <v>0.0334</v>
+        <v>-0.007900000000000001</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0842</v>
+        <v>0.0246</v>
       </c>
       <c r="H30" t="n">
-        <v>53.5</v>
+        <v>46.8</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>38.9</v>
       </c>
       <c r="J30" t="n">
-        <v>46.5</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="31">
@@ -5841,31 +5841,31 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="C31" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>99.8</v>
+        <v>99.7</v>
       </c>
       <c r="E31" t="n">
-        <v>0.003</v>
+        <v>0.006</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.0004</v>
+        <v>0.0062</v>
       </c>
       <c r="G31" t="n">
-        <v>0.3529</v>
+        <v>0.0448</v>
       </c>
       <c r="H31" t="n">
-        <v>94.09999999999999</v>
+        <v>67.2</v>
       </c>
       <c r="I31" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="J31" t="n">
         <v>0</v>
-      </c>
-      <c r="J31" t="n">
-        <v>5.9</v>
       </c>
     </row>
     <row r="32">
@@ -5875,31 +5875,31 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>12.5</v>
+        <v>4.3</v>
       </c>
       <c r="C32" t="n">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>85.40000000000001</v>
+        <v>95.7</v>
       </c>
       <c r="E32" t="n">
-        <v>0.27</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="F32" t="n">
-        <v>0.0109</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="G32" t="n">
-        <v>0.0771</v>
+        <v>0.0036</v>
       </c>
       <c r="H32" t="n">
-        <v>13.9</v>
+        <v>47.1</v>
       </c>
       <c r="I32" t="n">
-        <v>85.8</v>
+        <v>52.9</v>
       </c>
       <c r="J32" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -5909,31 +5909,31 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>4.2</v>
+        <v>1.1</v>
       </c>
       <c r="C33" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="D33" t="n">
-        <v>95.5</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="E33" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.027</v>
       </c>
       <c r="F33" t="n">
-        <v>0.008699999999999999</v>
+        <v>0.0275</v>
       </c>
       <c r="G33" t="n">
-        <v>0.0352</v>
+        <v>0.2013</v>
       </c>
       <c r="H33" t="n">
-        <v>39.9</v>
+        <v>51.7</v>
       </c>
       <c r="I33" t="n">
-        <v>59.2</v>
+        <v>48.3</v>
       </c>
       <c r="J33" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -6002,31 +6002,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1.2</v>
+        <v>0.7</v>
       </c>
       <c r="C39" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="D39" t="n">
-        <v>98.5</v>
+        <v>99.2</v>
       </c>
       <c r="E39" t="n">
-        <v>0.028</v>
+        <v>0.015</v>
       </c>
       <c r="F39" t="n">
-        <v>0.0339</v>
+        <v>0.0283</v>
       </c>
       <c r="G39" t="n">
-        <v>0.1023</v>
+        <v>0.0357</v>
       </c>
       <c r="H39" t="n">
-        <v>54.1</v>
+        <v>53</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>27.4</v>
       </c>
       <c r="J39" t="n">
-        <v>45.9</v>
+        <v>19.6</v>
       </c>
     </row>
     <row r="40">
@@ -6036,31 +6036,31 @@
         </is>
       </c>
       <c r="B40" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C40" t="n">
         <v>0.1</v>
       </c>
-      <c r="C40" t="n">
-        <v>0</v>
-      </c>
       <c r="D40" t="n">
-        <v>99.90000000000001</v>
+        <v>99.8</v>
       </c>
       <c r="E40" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.0056</v>
+        <v>0.0018</v>
       </c>
       <c r="G40" t="n">
-        <v>0.07140000000000001</v>
+        <v>0.1154</v>
       </c>
       <c r="H40" t="n">
-        <v>96.40000000000001</v>
+        <v>82.7</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>15.4</v>
       </c>
       <c r="J40" t="n">
-        <v>3.6</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="41">
@@ -6070,31 +6070,31 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>12.2</v>
+        <v>4.7</v>
       </c>
       <c r="C41" t="n">
-        <v>3.4</v>
+        <v>0.4</v>
       </c>
       <c r="D41" t="n">
-        <v>84.40000000000001</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="E41" t="n">
-        <v>0.279</v>
+        <v>0.098</v>
       </c>
       <c r="F41" t="n">
-        <v>0.0371</v>
+        <v>0.0324</v>
       </c>
       <c r="G41" t="n">
-        <v>0.1216</v>
+        <v>0.0428</v>
       </c>
       <c r="H41" t="n">
-        <v>13.3</v>
+        <v>39.5</v>
       </c>
       <c r="I41" t="n">
-        <v>86.2</v>
+        <v>60.5</v>
       </c>
       <c r="J41" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -6104,31 +6104,31 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>4.3</v>
+        <v>1.3</v>
       </c>
       <c r="C42" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="D42" t="n">
-        <v>95.40000000000001</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="E42" t="n">
-        <v>0.089</v>
+        <v>0.029</v>
       </c>
       <c r="F42" t="n">
-        <v>0.0298</v>
+        <v>0.0192</v>
       </c>
       <c r="G42" t="n">
-        <v>0.0267</v>
+        <v>0.1013</v>
       </c>
       <c r="H42" t="n">
-        <v>35.8</v>
+        <v>47.8</v>
       </c>
       <c r="I42" t="n">
-        <v>64.2</v>
+        <v>51.9</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="46">
@@ -6197,31 +6197,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
       <c r="C48" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="D48" t="n">
-        <v>98.09999999999999</v>
+        <v>98.8</v>
       </c>
       <c r="E48" t="n">
-        <v>0.035</v>
+        <v>0.022</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0174</v>
+        <v>0.0011</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0866</v>
+        <v>0.0798</v>
       </c>
       <c r="H48" t="n">
-        <v>51.6</v>
+        <v>46.1</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
+        <v>34.5</v>
       </c>
       <c r="J48" t="n">
-        <v>48.4</v>
+        <v>19.4</v>
       </c>
     </row>
     <row r="49">
@@ -6231,31 +6231,31 @@
         </is>
       </c>
       <c r="B49" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C49" t="n">
         <v>0.1</v>
       </c>
-      <c r="C49" t="n">
-        <v>0</v>
-      </c>
       <c r="D49" t="n">
-        <v>99.90000000000001</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="E49" t="n">
-        <v>0.002</v>
+        <v>0.007</v>
       </c>
       <c r="F49" t="n">
-        <v>0.0105</v>
+        <v>-0.0054</v>
       </c>
       <c r="G49" t="n">
-        <v>0.1262</v>
+        <v>0.1431</v>
       </c>
       <c r="H49" t="n">
-        <v>96.2</v>
+        <v>62.1</v>
       </c>
       <c r="I49" t="n">
-        <v>0</v>
+        <v>36.4</v>
       </c>
       <c r="J49" t="n">
-        <v>3.8</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="50">
@@ -6265,31 +6265,31 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>16</v>
+        <v>5.4</v>
       </c>
       <c r="C50" t="n">
-        <v>3.2</v>
+        <v>1.1</v>
       </c>
       <c r="D50" t="n">
-        <v>80.7</v>
+        <v>93.5</v>
       </c>
       <c r="E50" t="n">
-        <v>0.353</v>
+        <v>0.119</v>
       </c>
       <c r="F50" t="n">
-        <v>0.02</v>
+        <v>0.0165</v>
       </c>
       <c r="G50" t="n">
-        <v>0.096</v>
+        <v>0.0901</v>
       </c>
       <c r="H50" t="n">
-        <v>14.6</v>
+        <v>42.7</v>
       </c>
       <c r="I50" t="n">
-        <v>84.8</v>
+        <v>57.2</v>
       </c>
       <c r="J50" t="n">
-        <v>0.6</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="51">
@@ -6299,31 +6299,31 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>4.5</v>
+        <v>1.6</v>
       </c>
       <c r="C51" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="D51" t="n">
-        <v>95.09999999999999</v>
+        <v>97.8</v>
       </c>
       <c r="E51" t="n">
-        <v>0.094</v>
+        <v>0.038</v>
       </c>
       <c r="F51" t="n">
-        <v>0.007900000000000001</v>
+        <v>0.0125</v>
       </c>
       <c r="G51" t="n">
-        <v>0.0453</v>
+        <v>0.1689</v>
       </c>
       <c r="H51" t="n">
-        <v>40.6</v>
+        <v>45.6</v>
       </c>
       <c r="I51" t="n">
-        <v>58.9</v>
+        <v>53.9</v>
       </c>
       <c r="J51" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
strategy and baseline inventory model toggle, sigma fixed to mid-diff, gamma tuning
</commit_message>
<xml_diff>
--- a/sheets/fill_stats.xlsx
+++ b/sheets/fill_stats.xlsx
@@ -1670,28 +1670,28 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10.7</v>
+        <v>10.3</v>
       </c>
       <c r="C3" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="D3" t="n">
-        <v>88.8</v>
+        <v>89</v>
       </c>
       <c r="E3" t="n">
-        <v>0.219</v>
+        <v>0.212</v>
       </c>
       <c r="F3" t="n">
-        <v>0.6081</v>
+        <v>0.4017</v>
       </c>
       <c r="G3" t="n">
-        <v>0.024</v>
+        <v>0.0331</v>
       </c>
       <c r="H3" t="n">
-        <v>99.59999999999999</v>
+        <v>99.5</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="J3" t="n">
         <v>0.2</v>
@@ -1704,22 +1704,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10.1</v>
+        <v>10.2</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="D4" t="n">
-        <v>89.40000000000001</v>
+        <v>89.5</v>
       </c>
       <c r="E4" t="n">
         <v>0.207</v>
       </c>
       <c r="F4" t="n">
-        <v>0.5278</v>
+        <v>0.1244</v>
       </c>
       <c r="G4" t="n">
-        <v>0.022</v>
+        <v>0.0186</v>
       </c>
       <c r="H4" t="n">
         <v>99.8</v>
@@ -1865,28 +1865,28 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
       <c r="C12" t="n">
         <v>0.4</v>
       </c>
       <c r="D12" t="n">
-        <v>94.09999999999999</v>
+        <v>94</v>
       </c>
       <c r="E12" t="n">
-        <v>0.114</v>
+        <v>0.117</v>
       </c>
       <c r="F12" t="n">
-        <v>0.2342</v>
+        <v>0.1961</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0315</v>
+        <v>0.0317</v>
       </c>
       <c r="H12" t="n">
-        <v>98.59999999999999</v>
+        <v>98.7</v>
       </c>
       <c r="I12" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="J12" t="n">
         <v>1.1</v>
@@ -1899,28 +1899,28 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
       <c r="C13" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="D13" t="n">
         <v>94.2</v>
       </c>
       <c r="E13" t="n">
-        <v>0.11</v>
+        <v>0.112</v>
       </c>
       <c r="F13" t="n">
-        <v>0.284</v>
+        <v>0.3478</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0527</v>
+        <v>0.0357</v>
       </c>
       <c r="H13" t="n">
-        <v>99.59999999999999</v>
+        <v>99.5</v>
       </c>
       <c r="I13" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="J13" t="n">
         <v>0.1</v>
@@ -2060,22 +2060,22 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>5.6</v>
+        <v>5.5</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="D21" t="n">
         <v>93.40000000000001</v>
       </c>
       <c r="E21" t="n">
-        <v>0.122</v>
+        <v>0.121</v>
       </c>
       <c r="F21" t="n">
-        <v>0.5897</v>
+        <v>0.5357</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0805</v>
+        <v>0.0883</v>
       </c>
       <c r="H21" t="n">
         <v>99.09999999999999</v>
@@ -2084,7 +2084,7 @@
         <v>0.5</v>
       </c>
       <c r="J21" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="22">
@@ -2094,22 +2094,22 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
       <c r="C22" t="n">
-        <v>1.4</v>
+        <v>0.9</v>
       </c>
       <c r="D22" t="n">
-        <v>93.3</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>0.12</v>
+        <v>0.123</v>
       </c>
       <c r="F22" t="n">
-        <v>0.3716</v>
+        <v>0.7284</v>
       </c>
       <c r="G22" t="n">
-        <v>0.1129</v>
+        <v>0.0726</v>
       </c>
       <c r="H22" t="n">
         <v>99.59999999999999</v>
@@ -2258,28 +2258,28 @@
         <v>6.1</v>
       </c>
       <c r="C30" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D30" t="n">
         <v>93.8</v>
       </c>
       <c r="E30" t="n">
-        <v>0.122</v>
+        <v>0.123</v>
       </c>
       <c r="F30" t="n">
-        <v>0.5649</v>
+        <v>0.3586</v>
       </c>
       <c r="G30" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.0135</v>
       </c>
       <c r="H30" t="n">
-        <v>98.7</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="I30" t="n">
         <v>0.5</v>
       </c>
       <c r="J30" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="31">
@@ -2301,16 +2301,16 @@
         <v>0.117</v>
       </c>
       <c r="F31" t="n">
-        <v>0.5338000000000001</v>
+        <v>0.3848</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0131</v>
+        <v>0.0074</v>
       </c>
       <c r="H31" t="n">
         <v>99.40000000000001</v>
       </c>
       <c r="I31" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="J31" t="n">
         <v>0.4</v>
@@ -2450,31 +2450,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>8.199999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="C39" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="D39" t="n">
-        <v>90.3</v>
+        <v>90.2</v>
       </c>
       <c r="E39" t="n">
-        <v>0.178</v>
+        <v>0.181</v>
       </c>
       <c r="F39" t="n">
-        <v>0.4574</v>
+        <v>0.4254</v>
       </c>
       <c r="G39" t="n">
-        <v>0.08169999999999999</v>
+        <v>0.0868</v>
       </c>
       <c r="H39" t="n">
         <v>98.2</v>
       </c>
       <c r="I39" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="J39" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="40">
@@ -2484,28 +2484,28 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="C40" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="D40" t="n">
-        <v>91.2</v>
+        <v>91.3</v>
       </c>
       <c r="E40" t="n">
-        <v>0.164</v>
+        <v>0.161</v>
       </c>
       <c r="F40" t="n">
-        <v>0.4937</v>
+        <v>0.4273</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0697</v>
+        <v>0.073</v>
       </c>
       <c r="H40" t="n">
-        <v>98.90000000000001</v>
+        <v>98.8</v>
       </c>
       <c r="I40" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="J40" t="n">
         <v>0.3</v>
@@ -2645,10 +2645,10 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="C48" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="D48" t="n">
         <v>92.09999999999999</v>
@@ -2657,10 +2657,10 @@
         <v>0.151</v>
       </c>
       <c r="F48" t="n">
-        <v>0.4909</v>
+        <v>0.3835</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0452</v>
+        <v>0.0507</v>
       </c>
       <c r="H48" t="n">
         <v>98.90000000000001</v>
@@ -2679,10 +2679,10 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>6.8</v>
+        <v>6.9</v>
       </c>
       <c r="C49" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="D49" t="n">
         <v>92.5</v>
@@ -2691,16 +2691,16 @@
         <v>0.144</v>
       </c>
       <c r="F49" t="n">
-        <v>0.4422</v>
+        <v>0.4025</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0541</v>
+        <v>0.0415</v>
       </c>
       <c r="H49" t="n">
-        <v>99.5</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="I49" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="J49" t="n">
         <v>0.2</v>
@@ -2854,31 +2854,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17.6</v>
+        <v>14.7</v>
       </c>
       <c r="C3" t="n">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="D3" t="n">
-        <v>80.59999999999999</v>
+        <v>83.8</v>
       </c>
       <c r="E3" t="n">
-        <v>0.37</v>
+        <v>0.31</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0134</v>
+        <v>0.0113</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0492</v>
+        <v>0.0494</v>
       </c>
       <c r="H3" t="n">
-        <v>27.4</v>
+        <v>26.9</v>
       </c>
       <c r="I3" t="n">
-        <v>72.3</v>
+        <v>72.5</v>
       </c>
       <c r="J3" t="n">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="4">
@@ -2888,28 +2888,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7.7</v>
+        <v>6</v>
       </c>
       <c r="C4" t="n">
         <v>0.1</v>
       </c>
       <c r="D4" t="n">
-        <v>92.2</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>0.154</v>
+        <v>0.121</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0111</v>
+        <v>0.0058</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0043</v>
+        <v>0.0053</v>
       </c>
       <c r="H4" t="n">
-        <v>36.8</v>
+        <v>36.1</v>
       </c>
       <c r="I4" t="n">
-        <v>62.8</v>
+        <v>63.5</v>
       </c>
       <c r="J4" t="n">
         <v>0.4</v>
@@ -3049,31 +3049,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7.9</v>
+        <v>6.5</v>
       </c>
       <c r="C12" t="n">
-        <v>2.7</v>
+        <v>1.1</v>
       </c>
       <c r="D12" t="n">
-        <v>89.40000000000001</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>0.185</v>
+        <v>0.141</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.0476</v>
+        <v>-0.0232</v>
       </c>
       <c r="G12" t="n">
-        <v>0.148</v>
+        <v>0.08119999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>24.1</v>
+        <v>24</v>
       </c>
       <c r="I12" t="n">
         <v>75.7</v>
       </c>
       <c r="J12" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="13">
@@ -3083,31 +3083,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="C13" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="D13" t="n">
-        <v>96.59999999999999</v>
+        <v>97.2</v>
       </c>
       <c r="E13" t="n">
-        <v>0.063</v>
+        <v>0.054</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0377</v>
+        <v>-0.0152</v>
       </c>
       <c r="G13" t="n">
-        <v>0.08069999999999999</v>
+        <v>0.0197</v>
       </c>
       <c r="H13" t="n">
-        <v>41</v>
+        <v>40.6</v>
       </c>
       <c r="I13" t="n">
-        <v>58.7</v>
+        <v>59.4</v>
       </c>
       <c r="J13" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -3244,28 +3244,28 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>10.1</v>
+        <v>7.9</v>
       </c>
       <c r="C21" t="n">
         <v>0.2</v>
       </c>
       <c r="D21" t="n">
-        <v>89.7</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="E21" t="n">
-        <v>0.204</v>
+        <v>0.16</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.0149</v>
+        <v>-0.0055</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0097</v>
+        <v>0.0116</v>
       </c>
       <c r="H21" t="n">
-        <v>30.7</v>
+        <v>32.7</v>
       </c>
       <c r="I21" t="n">
-        <v>69.3</v>
+        <v>67.2</v>
       </c>
       <c r="J21" t="n">
         <v>0.1</v>
@@ -3278,28 +3278,28 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3.9</v>
+        <v>3.1</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>96.09999999999999</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>0.078</v>
+        <v>0.061</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.0186</v>
+        <v>-0.025</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0026</v>
+        <v>0.0032</v>
       </c>
       <c r="H22" t="n">
-        <v>42</v>
+        <v>42.9</v>
       </c>
       <c r="I22" t="n">
-        <v>58</v>
+        <v>57.1</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -3439,31 +3439,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>9.699999999999999</v>
+        <v>7.6</v>
       </c>
       <c r="C30" t="n">
-        <v>0.1</v>
+        <v>0.6</v>
       </c>
       <c r="D30" t="n">
-        <v>90.2</v>
+        <v>91.8</v>
       </c>
       <c r="E30" t="n">
-        <v>0.195</v>
+        <v>0.158</v>
       </c>
       <c r="F30" t="n">
-        <v>0.0259</v>
+        <v>0.0238</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0031</v>
+        <v>0.0369</v>
       </c>
       <c r="H30" t="n">
-        <v>28.5</v>
+        <v>28.4</v>
       </c>
       <c r="I30" t="n">
         <v>71.2</v>
       </c>
       <c r="J30" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="31">
@@ -3473,28 +3473,28 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3.1</v>
+        <v>2.8</v>
       </c>
       <c r="C31" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="D31" t="n">
-        <v>96.3</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="E31" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.057</v>
       </c>
       <c r="F31" t="n">
-        <v>0.0128</v>
+        <v>0.008</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0859</v>
+        <v>0.0224</v>
       </c>
       <c r="H31" t="n">
-        <v>36</v>
+        <v>35.5</v>
       </c>
       <c r="I31" t="n">
-        <v>64</v>
+        <v>64.5</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -3634,31 +3634,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>8.699999999999999</v>
+        <v>6.1</v>
       </c>
       <c r="C39" t="n">
-        <v>4.7</v>
+        <v>1.8</v>
       </c>
       <c r="D39" t="n">
-        <v>86.59999999999999</v>
+        <v>92</v>
       </c>
       <c r="E39" t="n">
-        <v>0.221</v>
+        <v>0.141</v>
       </c>
       <c r="F39" t="n">
-        <v>0.0336</v>
+        <v>0.0162</v>
       </c>
       <c r="G39" t="n">
-        <v>0.2133</v>
+        <v>0.13</v>
       </c>
       <c r="H39" t="n">
-        <v>20</v>
+        <v>20.5</v>
       </c>
       <c r="I39" t="n">
-        <v>80</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="40">
@@ -3668,28 +3668,28 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="C40" t="n">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="D40" t="n">
-        <v>96.09999999999999</v>
+        <v>97.3</v>
       </c>
       <c r="E40" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.052</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0277</v>
+        <v>0.0102</v>
       </c>
       <c r="G40" t="n">
-        <v>0.1288</v>
+        <v>0.0223</v>
       </c>
       <c r="H40" t="n">
-        <v>38.6</v>
+        <v>39.6</v>
       </c>
       <c r="I40" t="n">
-        <v>61.4</v>
+        <v>60.4</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -3829,31 +3829,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>10.8</v>
+        <v>8.6</v>
       </c>
       <c r="C48" t="n">
-        <v>1.9</v>
+        <v>1.1</v>
       </c>
       <c r="D48" t="n">
-        <v>87.3</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="E48" t="n">
-        <v>0.235</v>
+        <v>0.182</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0021</v>
+        <v>0.0045</v>
       </c>
       <c r="G48" t="n">
-        <v>0.08459999999999999</v>
+        <v>0.0618</v>
       </c>
       <c r="H48" t="n">
-        <v>26.2</v>
+        <v>26.7</v>
       </c>
       <c r="I48" t="n">
-        <v>73.59999999999999</v>
+        <v>73</v>
       </c>
       <c r="J48" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="49">
@@ -3863,31 +3863,31 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>4.1</v>
+        <v>3.4</v>
       </c>
       <c r="C49" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="D49" t="n">
-        <v>95.5</v>
+        <v>96.5</v>
       </c>
       <c r="E49" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="F49" t="n">
-        <v>-0.0009</v>
+        <v>-0.0032</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0605</v>
+        <v>0.0146</v>
       </c>
       <c r="H49" t="n">
-        <v>38.6</v>
+        <v>38.5</v>
       </c>
       <c r="I49" t="n">
-        <v>61.2</v>
+        <v>61.3</v>
       </c>
       <c r="J49" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="50">
@@ -4038,31 +4038,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.8</v>
+        <v>6.3</v>
       </c>
       <c r="C3" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="D3" t="n">
-        <v>91.8</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>0.16</v>
+        <v>0.127</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0256</v>
+        <v>0.0091</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0219</v>
+        <v>0.0103</v>
       </c>
       <c r="H3" t="n">
-        <v>68.8</v>
+        <v>62.7</v>
       </c>
       <c r="I3" t="n">
-        <v>30.2</v>
+        <v>35</v>
       </c>
       <c r="J3" t="n">
-        <v>0.9</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="4">
@@ -4072,31 +4072,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5.1</v>
+        <v>3.4</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="D4" t="n">
-        <v>94.59999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="E4" t="n">
-        <v>0.105</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0091</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0359</v>
+        <v>0.0273</v>
       </c>
       <c r="H4" t="n">
-        <v>78.2</v>
+        <v>72.7</v>
       </c>
       <c r="I4" t="n">
-        <v>21.3</v>
+        <v>25.9</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="5">
@@ -4233,31 +4233,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5.7</v>
+        <v>4.2</v>
       </c>
       <c r="C12" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="D12" t="n">
-        <v>92.90000000000001</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="E12" t="n">
-        <v>0.127</v>
+        <v>0.092</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0135</v>
+        <v>0.0179</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1096</v>
+        <v>0.0743</v>
       </c>
       <c r="H12" t="n">
-        <v>64.3</v>
+        <v>58.5</v>
       </c>
       <c r="I12" t="n">
-        <v>35</v>
+        <v>39.5</v>
       </c>
       <c r="J12" t="n">
-        <v>0.7</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="13">
@@ -4267,31 +4267,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3.8</v>
+        <v>2.3</v>
       </c>
       <c r="C13" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="D13" t="n">
-        <v>95.7</v>
+        <v>97.5</v>
       </c>
       <c r="E13" t="n">
-        <v>0.081</v>
+        <v>0.048</v>
       </c>
       <c r="F13" t="n">
-        <v>-0</v>
+        <v>0.0115</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0677</v>
+        <v>0.0384</v>
       </c>
       <c r="H13" t="n">
-        <v>75.09999999999999</v>
+        <v>67.7</v>
       </c>
       <c r="I13" t="n">
-        <v>24.4</v>
+        <v>31.3</v>
       </c>
       <c r="J13" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -4428,31 +4428,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6.7</v>
+        <v>5.7</v>
       </c>
       <c r="C21" t="n">
-        <v>1.3</v>
+        <v>0.7</v>
       </c>
       <c r="D21" t="n">
-        <v>92</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="E21" t="n">
-        <v>0.147</v>
+        <v>0.121</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0024</v>
+        <v>0.0068</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0878</v>
+        <v>0.0606</v>
       </c>
       <c r="H21" t="n">
-        <v>73.2</v>
+        <v>66.3</v>
       </c>
       <c r="I21" t="n">
-        <v>25.4</v>
+        <v>30.7</v>
       </c>
       <c r="J21" t="n">
-        <v>1.4</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="22">
@@ -4462,31 +4462,31 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4.9</v>
+        <v>3.5</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="D22" t="n">
-        <v>94.2</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>0.107</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.013</v>
+        <v>-0.0112</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0897</v>
+        <v>0.021</v>
       </c>
       <c r="H22" t="n">
-        <v>80.3</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="I22" t="n">
-        <v>18.6</v>
+        <v>24.7</v>
       </c>
       <c r="J22" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="23">
@@ -4623,31 +4623,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>9.800000000000001</v>
+        <v>6.5</v>
       </c>
       <c r="C30" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="D30" t="n">
-        <v>89.7</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="E30" t="n">
-        <v>0.201</v>
+        <v>0.132</v>
       </c>
       <c r="F30" t="n">
-        <v>0.0401</v>
+        <v>0.0195</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0287</v>
+        <v>0.0069</v>
       </c>
       <c r="H30" t="n">
-        <v>56.2</v>
+        <v>50.3</v>
       </c>
       <c r="I30" t="n">
-        <v>43.3</v>
+        <v>46.6</v>
       </c>
       <c r="J30" t="n">
-        <v>0.5</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="31">
@@ -4657,31 +4657,31 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3.8</v>
+        <v>2.2</v>
       </c>
       <c r="C31" t="n">
-        <v>0.9</v>
+        <v>0.1</v>
       </c>
       <c r="D31" t="n">
-        <v>95.3</v>
+        <v>97.7</v>
       </c>
       <c r="E31" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.046</v>
       </c>
       <c r="F31" t="n">
-        <v>-0.0199</v>
+        <v>0.0234</v>
       </c>
       <c r="G31" t="n">
-        <v>0.1014</v>
+        <v>0.0231</v>
       </c>
       <c r="H31" t="n">
-        <v>62.1</v>
+        <v>60</v>
       </c>
       <c r="I31" t="n">
-        <v>37.9</v>
+        <v>39.8</v>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="32">
@@ -4818,31 +4818,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5.9</v>
+        <v>4.6</v>
       </c>
       <c r="C39" t="n">
-        <v>1.4</v>
+        <v>0.5</v>
       </c>
       <c r="D39" t="n">
-        <v>92.7</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="E39" t="n">
-        <v>0.133</v>
+        <v>0.097</v>
       </c>
       <c r="F39" t="n">
-        <v>0.008699999999999999</v>
+        <v>-0.0005</v>
       </c>
       <c r="G39" t="n">
-        <v>0.1037</v>
+        <v>0.0518</v>
       </c>
       <c r="H39" t="n">
-        <v>55.6</v>
+        <v>47.9</v>
       </c>
       <c r="I39" t="n">
-        <v>43.6</v>
+        <v>48.8</v>
       </c>
       <c r="J39" t="n">
-        <v>0.8</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="40">
@@ -4852,31 +4852,31 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>3.7</v>
+        <v>2.4</v>
       </c>
       <c r="C40" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>95.8</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="E40" t="n">
-        <v>0.079</v>
+        <v>0.047</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0114</v>
+        <v>-0.0128</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0675</v>
+        <v>0.0041</v>
       </c>
       <c r="H40" t="n">
-        <v>68.3</v>
+        <v>59.8</v>
       </c>
       <c r="I40" t="n">
-        <v>30.6</v>
+        <v>39.2</v>
       </c>
       <c r="J40" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -5013,31 +5013,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>7.2</v>
+        <v>5.5</v>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="D48" t="n">
-        <v>91.8</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="E48" t="n">
-        <v>0.153</v>
+        <v>0.114</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0181</v>
+        <v>0.0106</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0703</v>
+        <v>0.0408</v>
       </c>
       <c r="H48" t="n">
-        <v>63.5</v>
+        <v>57.4</v>
       </c>
       <c r="I48" t="n">
-        <v>35.7</v>
+        <v>39.9</v>
       </c>
       <c r="J48" t="n">
-        <v>0.9</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="49">
@@ -5047,31 +5047,31 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>4.2</v>
+        <v>2.7</v>
       </c>
       <c r="C49" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="D49" t="n">
-        <v>95.09999999999999</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="E49" t="n">
-        <v>0.091</v>
+        <v>0.056</v>
       </c>
       <c r="F49" t="n">
-        <v>-0.0025</v>
+        <v>0.0002</v>
       </c>
       <c r="G49" t="n">
-        <v>0.07240000000000001</v>
+        <v>0.0228</v>
       </c>
       <c r="H49" t="n">
-        <v>73.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="I49" t="n">
-        <v>26</v>
+        <v>31.1</v>
       </c>
       <c r="J49" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -5222,31 +5222,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>97.5</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>0.046</v>
+        <v>0.051</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.0352</v>
+        <v>-0.0014</v>
       </c>
       <c r="G3" t="n">
-        <v>0.06909999999999999</v>
+        <v>0.0056</v>
       </c>
       <c r="H3" t="n">
-        <v>47.8</v>
+        <v>52.5</v>
       </c>
       <c r="I3" t="n">
-        <v>33.9</v>
+        <v>34.1</v>
       </c>
       <c r="J3" t="n">
-        <v>18.3</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="4">
@@ -5256,31 +5256,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>99.09999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>0.016</v>
+        <v>0.017</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0451</v>
+        <v>-0.0039</v>
       </c>
       <c r="G4" t="n">
-        <v>0.116</v>
+        <v>0.0103</v>
       </c>
       <c r="H4" t="n">
-        <v>57.5</v>
+        <v>58.8</v>
       </c>
       <c r="I4" t="n">
-        <v>40.3</v>
+        <v>38.7</v>
       </c>
       <c r="J4" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="5">
@@ -5417,31 +5417,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="C12" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
         <v>99.09999999999999</v>
       </c>
       <c r="E12" t="n">
-        <v>0.015</v>
+        <v>0.018</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0217</v>
+        <v>0.005</v>
       </c>
       <c r="G12" t="n">
-        <v>0.1786</v>
+        <v>0.01</v>
       </c>
       <c r="H12" t="n">
-        <v>41.1</v>
+        <v>42</v>
       </c>
       <c r="I12" t="n">
-        <v>35.7</v>
+        <v>39</v>
       </c>
       <c r="J12" t="n">
-        <v>23.2</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13">
@@ -5454,28 +5454,28 @@
         <v>0.2</v>
       </c>
       <c r="C13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
         <v>99.8</v>
       </c>
       <c r="E13" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0234</v>
+        <v>0.0115</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1304</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>54.3</v>
+        <v>57.4</v>
       </c>
       <c r="I13" t="n">
-        <v>43.5</v>
+        <v>42.6</v>
       </c>
       <c r="J13" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -5612,31 +5612,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="C21" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>99</v>
       </c>
       <c r="E21" t="n">
-        <v>0.018</v>
+        <v>0.021</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.0016</v>
+        <v>-0.012</v>
       </c>
       <c r="G21" t="n">
-        <v>0.09089999999999999</v>
+        <v>0.0131</v>
       </c>
       <c r="H21" t="n">
-        <v>39.4</v>
+        <v>44.1</v>
       </c>
       <c r="I21" t="n">
-        <v>36.4</v>
+        <v>37.6</v>
       </c>
       <c r="J21" t="n">
-        <v>24.2</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="22">
@@ -5646,10 +5646,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="C22" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>99.7</v>
@@ -5658,19 +5658,19 @@
         <v>0.005</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.0133</v>
+        <v>-0.0075</v>
       </c>
       <c r="G22" t="n">
-        <v>0.3091</v>
+        <v>0.0159</v>
       </c>
       <c r="H22" t="n">
-        <v>58.2</v>
+        <v>49.2</v>
       </c>
       <c r="I22" t="n">
-        <v>41.8</v>
+        <v>49.2</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="23">
@@ -5807,31 +5807,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>99.09999999999999</v>
+        <v>99</v>
       </c>
       <c r="E30" t="n">
-        <v>0.018</v>
+        <v>0.02</v>
       </c>
       <c r="F30" t="n">
-        <v>-0.007900000000000001</v>
+        <v>0.0067</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0246</v>
+        <v>0.0046</v>
       </c>
       <c r="H30" t="n">
-        <v>46.8</v>
+        <v>48.4</v>
       </c>
       <c r="I30" t="n">
-        <v>38.9</v>
+        <v>38.8</v>
       </c>
       <c r="J30" t="n">
-        <v>14.3</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="31">
@@ -5850,19 +5850,19 @@
         <v>99.7</v>
       </c>
       <c r="E31" t="n">
-        <v>0.006</v>
+        <v>0.007</v>
       </c>
       <c r="F31" t="n">
-        <v>0.0062</v>
+        <v>0.0032</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0448</v>
+        <v>0.0127</v>
       </c>
       <c r="H31" t="n">
-        <v>67.2</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="I31" t="n">
-        <v>32.8</v>
+        <v>30.4</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -6002,31 +6002,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="C39" t="n">
         <v>0.1</v>
       </c>
       <c r="D39" t="n">
-        <v>99.2</v>
+        <v>99</v>
       </c>
       <c r="E39" t="n">
-        <v>0.015</v>
+        <v>0.019</v>
       </c>
       <c r="F39" t="n">
-        <v>0.0283</v>
+        <v>0.0151</v>
       </c>
       <c r="G39" t="n">
-        <v>0.0357</v>
+        <v>0.0419</v>
       </c>
       <c r="H39" t="n">
-        <v>53</v>
+        <v>49.3</v>
       </c>
       <c r="I39" t="n">
-        <v>27.4</v>
+        <v>36.7</v>
       </c>
       <c r="J39" t="n">
-        <v>19.6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="40">
@@ -6039,7 +6039,7 @@
         <v>0.2</v>
       </c>
       <c r="C40" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D40" t="n">
         <v>99.8</v>
@@ -6048,19 +6048,19 @@
         <v>0.004</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0018</v>
+        <v>0.0054</v>
       </c>
       <c r="G40" t="n">
-        <v>0.1154</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="H40" t="n">
-        <v>82.7</v>
+        <v>84.8</v>
       </c>
       <c r="I40" t="n">
-        <v>15.4</v>
+        <v>13</v>
       </c>
       <c r="J40" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="41">
@@ -6197,31 +6197,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="C48" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D48" t="n">
-        <v>98.8</v>
+        <v>98.7</v>
       </c>
       <c r="E48" t="n">
-        <v>0.022</v>
+        <v>0.026</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0011</v>
+        <v>0.0027</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0798</v>
+        <v>0.015</v>
       </c>
       <c r="H48" t="n">
-        <v>46.1</v>
+        <v>48.5</v>
       </c>
       <c r="I48" t="n">
-        <v>34.5</v>
+        <v>36.5</v>
       </c>
       <c r="J48" t="n">
-        <v>19.4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="49">
@@ -6231,31 +6231,31 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="C49" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D49" t="n">
         <v>99.59999999999999</v>
       </c>
       <c r="E49" t="n">
-        <v>0.007</v>
+        <v>0.008</v>
       </c>
       <c r="F49" t="n">
-        <v>-0.0054</v>
+        <v>0.0017</v>
       </c>
       <c r="G49" t="n">
-        <v>0.1431</v>
+        <v>0.0252</v>
       </c>
       <c r="H49" t="n">
-        <v>62.1</v>
+        <v>61.9</v>
       </c>
       <c r="I49" t="n">
-        <v>36.4</v>
+        <v>36.5</v>
       </c>
       <c r="J49" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="50">

</xml_diff>

<commit_message>
fixed sigma lookahead, documentation throughout
</commit_message>
<xml_diff>
--- a/sheets/fill_stats.xlsx
+++ b/sheets/fill_stats.xlsx
@@ -1716,10 +1716,10 @@
         <v>0.207</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1244</v>
+        <v>0.1161</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0186</v>
+        <v>0.018</v>
       </c>
       <c r="H4" t="n">
         <v>99.8</v>
@@ -2462,7 +2462,7 @@
         <v>0.181</v>
       </c>
       <c r="F39" t="n">
-        <v>0.4254</v>
+        <v>0.4255</v>
       </c>
       <c r="G39" t="n">
         <v>0.0868</v>
@@ -2487,19 +2487,19 @@
         <v>7.5</v>
       </c>
       <c r="C40" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="D40" t="n">
-        <v>91.3</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="E40" t="n">
         <v>0.161</v>
       </c>
       <c r="F40" t="n">
-        <v>0.4273</v>
+        <v>0.4282</v>
       </c>
       <c r="G40" t="n">
-        <v>0.073</v>
+        <v>0.0716</v>
       </c>
       <c r="H40" t="n">
         <v>98.8</v>
@@ -2691,10 +2691,10 @@
         <v>0.144</v>
       </c>
       <c r="F49" t="n">
-        <v>0.4025</v>
+        <v>0.401</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0415</v>
+        <v>0.0411</v>
       </c>
       <c r="H49" t="n">
         <v>99.40000000000001</v>
@@ -4038,31 +4038,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6.3</v>
+        <v>7.1</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>93.59999999999999</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>0.127</v>
+        <v>0.142</v>
       </c>
       <c r="F3" t="n">
         <v>0.0091</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0103</v>
+        <v>0.0024</v>
       </c>
       <c r="H3" t="n">
-        <v>62.7</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="I3" t="n">
-        <v>35</v>
+        <v>33.5</v>
       </c>
       <c r="J3" t="n">
-        <v>2.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="4">
@@ -4072,31 +4072,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="D4" t="n">
-        <v>96.5</v>
+        <v>95.8</v>
       </c>
       <c r="E4" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.082</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0041</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0273</v>
+        <v>0.0334</v>
       </c>
       <c r="H4" t="n">
-        <v>72.7</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>25.9</v>
+        <v>25.1</v>
       </c>
       <c r="J4" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -4233,31 +4233,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4.2</v>
+        <v>4.9</v>
       </c>
       <c r="C12" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="D12" t="n">
-        <v>95.09999999999999</v>
+        <v>94.3</v>
       </c>
       <c r="E12" t="n">
-        <v>0.092</v>
+        <v>0.106</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0179</v>
+        <v>0.0196</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0743</v>
+        <v>0.07820000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>58.5</v>
+        <v>60.1</v>
       </c>
       <c r="I12" t="n">
-        <v>39.5</v>
+        <v>38.5</v>
       </c>
       <c r="J12" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="13">
@@ -4267,28 +4267,28 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2.3</v>
+        <v>2.9</v>
       </c>
       <c r="C13" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="D13" t="n">
-        <v>97.5</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="E13" t="n">
-        <v>0.048</v>
+        <v>0.06</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0115</v>
+        <v>0.0026</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0384</v>
+        <v>0.0195</v>
       </c>
       <c r="H13" t="n">
-        <v>67.7</v>
+        <v>70</v>
       </c>
       <c r="I13" t="n">
-        <v>31.3</v>
+        <v>29</v>
       </c>
       <c r="J13" t="n">
         <v>1</v>
@@ -4428,31 +4428,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>5.7</v>
+        <v>6.3</v>
       </c>
       <c r="C21" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>93.59999999999999</v>
+        <v>92.8</v>
       </c>
       <c r="E21" t="n">
-        <v>0.121</v>
+        <v>0.135</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0068</v>
+        <v>-0.0049</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0606</v>
+        <v>0.0709</v>
       </c>
       <c r="H21" t="n">
-        <v>66.3</v>
+        <v>70.8</v>
       </c>
       <c r="I21" t="n">
-        <v>30.7</v>
+        <v>27.3</v>
       </c>
       <c r="J21" t="n">
-        <v>2.9</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="22">
@@ -4462,28 +4462,28 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3.5</v>
+        <v>4.2</v>
       </c>
       <c r="C22" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="D22" t="n">
-        <v>96.40000000000001</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.0112</v>
+        <v>-0.018</v>
       </c>
       <c r="G22" t="n">
-        <v>0.021</v>
+        <v>0.0461</v>
       </c>
       <c r="H22" t="n">
-        <v>74.09999999999999</v>
+        <v>76.8</v>
       </c>
       <c r="I22" t="n">
-        <v>24.7</v>
+        <v>21.9</v>
       </c>
       <c r="J22" t="n">
         <v>1.3</v>
@@ -4623,31 +4623,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>6.5</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="C30" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>93.40000000000001</v>
+        <v>91.7</v>
       </c>
       <c r="E30" t="n">
-        <v>0.132</v>
+        <v>0.166</v>
       </c>
       <c r="F30" t="n">
-        <v>0.0195</v>
+        <v>0.02</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0069</v>
+        <v>0.0007</v>
       </c>
       <c r="H30" t="n">
-        <v>50.3</v>
+        <v>53.1</v>
       </c>
       <c r="I30" t="n">
-        <v>46.6</v>
+        <v>45.1</v>
       </c>
       <c r="J30" t="n">
-        <v>3.1</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="31">
@@ -4657,31 +4657,31 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2.2</v>
+        <v>3.1</v>
       </c>
       <c r="C31" t="n">
         <v>0.1</v>
       </c>
       <c r="D31" t="n">
-        <v>97.7</v>
+        <v>96.8</v>
       </c>
       <c r="E31" t="n">
-        <v>0.046</v>
+        <v>0.063</v>
       </c>
       <c r="F31" t="n">
-        <v>0.0234</v>
+        <v>0.0183</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0231</v>
+        <v>0.0202</v>
       </c>
       <c r="H31" t="n">
-        <v>60</v>
+        <v>57.5</v>
       </c>
       <c r="I31" t="n">
-        <v>39.8</v>
+        <v>42.5</v>
       </c>
       <c r="J31" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -4818,31 +4818,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>4.6</v>
+        <v>5.3</v>
       </c>
       <c r="C39" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="D39" t="n">
-        <v>94.90000000000001</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="E39" t="n">
-        <v>0.097</v>
+        <v>0.113</v>
       </c>
       <c r="F39" t="n">
-        <v>-0.0005</v>
+        <v>0.0026</v>
       </c>
       <c r="G39" t="n">
-        <v>0.0518</v>
+        <v>0.0516</v>
       </c>
       <c r="H39" t="n">
-        <v>47.9</v>
+        <v>51.4</v>
       </c>
       <c r="I39" t="n">
-        <v>48.8</v>
+        <v>46.1</v>
       </c>
       <c r="J39" t="n">
-        <v>3.2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="40">
@@ -4852,31 +4852,31 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
       <c r="C40" t="n">
         <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>97.59999999999999</v>
+        <v>97</v>
       </c>
       <c r="E40" t="n">
-        <v>0.047</v>
+        <v>0.059</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.0128</v>
+        <v>-0.0196</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0041</v>
+        <v>0.0016</v>
       </c>
       <c r="H40" t="n">
-        <v>59.8</v>
+        <v>65</v>
       </c>
       <c r="I40" t="n">
-        <v>39.2</v>
+        <v>34.2</v>
       </c>
       <c r="J40" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="41">
@@ -5013,31 +5013,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>5.5</v>
+        <v>6.4</v>
       </c>
       <c r="C48" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="D48" t="n">
-        <v>94.09999999999999</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="E48" t="n">
-        <v>0.114</v>
+        <v>0.132</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0106</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0408</v>
+        <v>0.0407</v>
       </c>
       <c r="H48" t="n">
-        <v>57.4</v>
+        <v>60.2</v>
       </c>
       <c r="I48" t="n">
-        <v>39.9</v>
+        <v>38</v>
       </c>
       <c r="J48" t="n">
-        <v>2.7</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="49">
@@ -5047,31 +5047,31 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2.7</v>
+        <v>3.4</v>
       </c>
       <c r="C49" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D49" t="n">
-        <v>97.09999999999999</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="E49" t="n">
-        <v>0.056</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="F49" t="n">
-        <v>0.0002</v>
+        <v>-0.0041</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0228</v>
+        <v>0.0242</v>
       </c>
       <c r="H49" t="n">
-        <v>67.8</v>
+        <v>69.5</v>
       </c>
       <c r="I49" t="n">
-        <v>31.1</v>
+        <v>29.7</v>
       </c>
       <c r="J49" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="50">

</xml_diff>

<commit_message>
changed gamma and q
</commit_message>
<xml_diff>
--- a/sheets/fill_stats.xlsx
+++ b/sheets/fill_stats.xlsx
@@ -486,31 +486,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>25.6</v>
+        <v>18.6</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>73.5</v>
+        <v>81.40000000000001</v>
       </c>
       <c r="E3" t="n">
-        <v>0.52</v>
+        <v>0.372</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0264</v>
+        <v>0.0172</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0174</v>
+        <v>0.0011</v>
       </c>
       <c r="H3" t="n">
-        <v>50.5</v>
+        <v>49.4</v>
       </c>
       <c r="I3" t="n">
-        <v>23.2</v>
+        <v>18.5</v>
       </c>
       <c r="J3" t="n">
-        <v>26.3</v>
+        <v>32.1</v>
       </c>
     </row>
     <row r="4">
@@ -520,28 +520,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8.1</v>
+        <v>3.1</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>91.90000000000001</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>0.162</v>
+        <v>0.061</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0526</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
       <c r="H4" t="n">
-        <v>64.8</v>
+        <v>67.90000000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>31.1</v>
+        <v>28</v>
       </c>
       <c r="J4" t="n">
         <v>4.1</v>
@@ -681,31 +681,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9</v>
+        <v>6.1</v>
       </c>
       <c r="C12" t="n">
-        <v>1.2</v>
+        <v>0.2</v>
       </c>
       <c r="D12" t="n">
-        <v>89.8</v>
+        <v>93.8</v>
       </c>
       <c r="E12" t="n">
-        <v>0.193</v>
+        <v>0.123</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0184</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0617</v>
+        <v>0.0132</v>
       </c>
       <c r="H12" t="n">
-        <v>46.8</v>
+        <v>45.6</v>
       </c>
       <c r="I12" t="n">
-        <v>18.3</v>
+        <v>23.4</v>
       </c>
       <c r="J12" t="n">
-        <v>34.9</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13">
@@ -715,31 +715,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.4</v>
+        <v>0.5</v>
       </c>
       <c r="C13" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>98.40000000000001</v>
+        <v>99.5</v>
       </c>
       <c r="E13" t="n">
-        <v>0.03</v>
+        <v>0.011</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0314</v>
+        <v>0.0037</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0801</v>
+        <v>0.0167</v>
       </c>
       <c r="H13" t="n">
-        <v>70.3</v>
+        <v>77.5</v>
       </c>
       <c r="I13" t="n">
-        <v>27.3</v>
+        <v>20</v>
       </c>
       <c r="J13" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="14">
@@ -876,31 +876,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>10.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="C21" t="n">
-        <v>1.5</v>
+        <v>0.4</v>
       </c>
       <c r="D21" t="n">
-        <v>87.8</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="E21" t="n">
-        <v>0.229</v>
+        <v>0.169</v>
       </c>
       <c r="F21" t="n">
-        <v>0.0375</v>
+        <v>0.04</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0673</v>
+        <v>0.0215</v>
       </c>
       <c r="H21" t="n">
-        <v>48.5</v>
+        <v>48.9</v>
       </c>
       <c r="I21" t="n">
-        <v>15.9</v>
+        <v>18.1</v>
       </c>
       <c r="J21" t="n">
-        <v>35.7</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22">
@@ -910,31 +910,31 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1.5</v>
+        <v>0.8</v>
       </c>
       <c r="C22" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>98.3</v>
+        <v>99.2</v>
       </c>
       <c r="E22" t="n">
-        <v>0.032</v>
+        <v>0.016</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.07829999999999999</v>
+        <v>-0.0207</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0592</v>
+        <v>0.0055</v>
       </c>
       <c r="H22" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I22" t="n">
-        <v>21.1</v>
+        <v>20.4</v>
       </c>
       <c r="J22" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="23">
@@ -1071,31 +1071,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>10</v>
+        <v>6.4</v>
       </c>
       <c r="C30" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="D30" t="n">
-        <v>89.59999999999999</v>
+        <v>93.5</v>
       </c>
       <c r="E30" t="n">
-        <v>0.204</v>
+        <v>0.129</v>
       </c>
       <c r="F30" t="n">
-        <v>0.004</v>
+        <v>0.0141</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0218</v>
+        <v>0.0102</v>
       </c>
       <c r="H30" t="n">
-        <v>48.9</v>
+        <v>47.5</v>
       </c>
       <c r="I30" t="n">
-        <v>19.1</v>
+        <v>21</v>
       </c>
       <c r="J30" t="n">
-        <v>32.1</v>
+        <v>31.6</v>
       </c>
     </row>
     <row r="31">
@@ -1105,31 +1105,31 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1.6</v>
+        <v>0.7</v>
       </c>
       <c r="C31" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>98.09999999999999</v>
+        <v>99.3</v>
       </c>
       <c r="E31" t="n">
-        <v>0.035</v>
+        <v>0.013</v>
       </c>
       <c r="F31" t="n">
-        <v>0.0171</v>
+        <v>-0.0028</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0718</v>
+        <v>0.0066</v>
       </c>
       <c r="H31" t="n">
-        <v>73.8</v>
+        <v>74.2</v>
       </c>
       <c r="I31" t="n">
-        <v>25.1</v>
+        <v>22.5</v>
       </c>
       <c r="J31" t="n">
-        <v>1</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="32">
@@ -1266,31 +1266,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>7.9</v>
+        <v>5.4</v>
       </c>
       <c r="C39" t="n">
-        <v>1.3</v>
+        <v>0.2</v>
       </c>
       <c r="D39" t="n">
-        <v>90.8</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="E39" t="n">
-        <v>0.172</v>
+        <v>0.11</v>
       </c>
       <c r="F39" t="n">
-        <v>0.0212</v>
+        <v>0.0139</v>
       </c>
       <c r="G39" t="n">
-        <v>0.0764</v>
+        <v>0.0203</v>
       </c>
       <c r="H39" t="n">
-        <v>48</v>
+        <v>46.3</v>
       </c>
       <c r="I39" t="n">
-        <v>17.6</v>
+        <v>22.6</v>
       </c>
       <c r="J39" t="n">
-        <v>34.5</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="40">
@@ -1300,31 +1300,31 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="C40" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>98.7</v>
+        <v>99.5</v>
       </c>
       <c r="E40" t="n">
-        <v>0.022</v>
+        <v>0.01</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.025</v>
+        <v>-0.0187</v>
       </c>
       <c r="G40" t="n">
-        <v>0.1592</v>
+        <v>0</v>
       </c>
       <c r="H40" t="n">
-        <v>77.09999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="I40" t="n">
-        <v>22.9</v>
+        <v>18.2</v>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="41">
@@ -1461,31 +1461,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>12.6</v>
+        <v>8.9</v>
       </c>
       <c r="C48" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
       <c r="D48" t="n">
-        <v>86.3</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="E48" t="n">
-        <v>0.264</v>
+        <v>0.181</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0215</v>
+        <v>0.0186</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0489</v>
+        <v>0.0132</v>
       </c>
       <c r="H48" t="n">
-        <v>48.9</v>
+        <v>48</v>
       </c>
       <c r="I48" t="n">
-        <v>19.6</v>
+        <v>20.1</v>
       </c>
       <c r="J48" t="n">
-        <v>31.4</v>
+        <v>31.9</v>
       </c>
     </row>
     <row r="49">
@@ -1495,31 +1495,31 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>2.7</v>
+        <v>1.1</v>
       </c>
       <c r="C49" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>97.09999999999999</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="E49" t="n">
-        <v>0.056</v>
+        <v>0.022</v>
       </c>
       <c r="F49" t="n">
-        <v>-0.0004</v>
+        <v>-0.0059</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0741</v>
+        <v>0.0064</v>
       </c>
       <c r="H49" t="n">
-        <v>69.2</v>
+        <v>72.3</v>
       </c>
       <c r="I49" t="n">
-        <v>28</v>
+        <v>24.5</v>
       </c>
       <c r="J49" t="n">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="50">
@@ -1670,31 +1670,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10.3</v>
+        <v>1.3</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="D3" t="n">
-        <v>89</v>
+        <v>98.7</v>
       </c>
       <c r="E3" t="n">
-        <v>0.212</v>
+        <v>0.026</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4017</v>
+        <v>-0.2865</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0331</v>
+        <v>0.0246</v>
       </c>
       <c r="H3" t="n">
-        <v>99.5</v>
+        <v>96.8</v>
       </c>
       <c r="I3" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="4">
@@ -1704,31 +1704,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10.2</v>
+        <v>0.4</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>89.5</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>0.207</v>
+        <v>0.008</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1161</v>
+        <v>0.0157</v>
       </c>
       <c r="G4" t="n">
-        <v>0.018</v>
+        <v>0.0217</v>
       </c>
       <c r="H4" t="n">
-        <v>99.8</v>
+        <v>100</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1865,31 +1865,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5.7</v>
+        <v>0.3</v>
       </c>
       <c r="C12" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>94</v>
+        <v>99.7</v>
       </c>
       <c r="E12" t="n">
-        <v>0.117</v>
+        <v>0.007</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1961</v>
+        <v>0.0177</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0317</v>
+        <v>0.0263</v>
       </c>
       <c r="H12" t="n">
-        <v>98.7</v>
+        <v>94.7</v>
       </c>
       <c r="I12" t="n">
-        <v>0.2</v>
+        <v>1.3</v>
       </c>
       <c r="J12" t="n">
-        <v>1.1</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="13">
@@ -1899,31 +1899,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5.4</v>
+        <v>0.1</v>
       </c>
       <c r="C13" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>94.2</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="E13" t="n">
-        <v>0.112</v>
+        <v>0.003</v>
       </c>
       <c r="F13" t="n">
-        <v>0.3478</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0357</v>
+        <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>99.5</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="I13" t="n">
-        <v>0.4</v>
+        <v>2.9</v>
       </c>
       <c r="J13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2060,31 +2060,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>5.5</v>
+        <v>1.3</v>
       </c>
       <c r="C21" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>93.40000000000001</v>
+        <v>98.7</v>
       </c>
       <c r="E21" t="n">
-        <v>0.121</v>
+        <v>0.027</v>
       </c>
       <c r="F21" t="n">
-        <v>0.5357</v>
+        <v>0.0325</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0883</v>
+        <v>0.0034</v>
       </c>
       <c r="H21" t="n">
-        <v>99.09999999999999</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="J21" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -2094,31 +2094,31 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>5.7</v>
+        <v>1.1</v>
       </c>
       <c r="C22" t="n">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>93.40000000000001</v>
+        <v>98.90000000000001</v>
       </c>
       <c r="E22" t="n">
-        <v>0.123</v>
+        <v>0.023</v>
       </c>
       <c r="F22" t="n">
-        <v>0.7284</v>
+        <v>0.0004</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0726</v>
+        <v>0.004</v>
       </c>
       <c r="H22" t="n">
-        <v>99.59999999999999</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="I22" t="n">
-        <v>0.2</v>
+        <v>1.6</v>
       </c>
       <c r="J22" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -2255,31 +2255,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>6.1</v>
+        <v>0.5</v>
       </c>
       <c r="C30" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>93.8</v>
+        <v>99.5</v>
       </c>
       <c r="E30" t="n">
-        <v>0.123</v>
+        <v>0.01</v>
       </c>
       <c r="F30" t="n">
-        <v>0.3586</v>
+        <v>-0.0951</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0135</v>
+        <v>0.0357</v>
       </c>
       <c r="H30" t="n">
-        <v>98.90000000000001</v>
+        <v>98.2</v>
       </c>
       <c r="I30" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="J30" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="31">
@@ -2289,31 +2289,31 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>5.8</v>
+        <v>0.3</v>
       </c>
       <c r="C31" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>94.09999999999999</v>
+        <v>99.7</v>
       </c>
       <c r="E31" t="n">
-        <v>0.117</v>
+        <v>0.006</v>
       </c>
       <c r="F31" t="n">
-        <v>0.3848</v>
+        <v>0.0463</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0074</v>
+        <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>99.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="I31" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -2450,31 +2450,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>8.300000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="C39" t="n">
-        <v>1.6</v>
+        <v>0.1</v>
       </c>
       <c r="D39" t="n">
-        <v>90.2</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="E39" t="n">
-        <v>0.181</v>
+        <v>0.018</v>
       </c>
       <c r="F39" t="n">
-        <v>0.4255</v>
+        <v>0.0731</v>
       </c>
       <c r="G39" t="n">
-        <v>0.0868</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="H39" t="n">
-        <v>98.2</v>
+        <v>95</v>
       </c>
       <c r="I39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>0.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40">
@@ -2484,31 +2484,31 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>7.5</v>
+        <v>0.6</v>
       </c>
       <c r="C40" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>91.40000000000001</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E40" t="n">
-        <v>0.161</v>
+        <v>0.012</v>
       </c>
       <c r="F40" t="n">
-        <v>0.4282</v>
+        <v>-0.0555</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0716</v>
+        <v>0.0074</v>
       </c>
       <c r="H40" t="n">
-        <v>98.8</v>
+        <v>97</v>
       </c>
       <c r="I40" t="n">
-        <v>0.9</v>
+        <v>2.2</v>
       </c>
       <c r="J40" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="41">
@@ -2645,31 +2645,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>7.1</v>
+        <v>0.9</v>
       </c>
       <c r="C48" t="n">
-        <v>0.8</v>
+        <v>0.1</v>
       </c>
       <c r="D48" t="n">
-        <v>92.09999999999999</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="E48" t="n">
-        <v>0.151</v>
+        <v>0.017</v>
       </c>
       <c r="F48" t="n">
-        <v>0.3835</v>
+        <v>-0.0517</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0507</v>
+        <v>0.032</v>
       </c>
       <c r="H48" t="n">
-        <v>98.90000000000001</v>
+        <v>97</v>
       </c>
       <c r="I48" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="J48" t="n">
-        <v>0.6</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="49">
@@ -2679,28 +2679,28 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>6.9</v>
+        <v>0.5</v>
       </c>
       <c r="C49" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>92.5</v>
+        <v>99.5</v>
       </c>
       <c r="E49" t="n">
-        <v>0.144</v>
+        <v>0.01</v>
       </c>
       <c r="F49" t="n">
-        <v>0.401</v>
+        <v>0.003</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0411</v>
+        <v>0.0066</v>
       </c>
       <c r="H49" t="n">
-        <v>99.40000000000001</v>
+        <v>98.5</v>
       </c>
       <c r="I49" t="n">
-        <v>0.4</v>
+        <v>1.4</v>
       </c>
       <c r="J49" t="n">
         <v>0.2</v>
@@ -2854,31 +2854,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14.7</v>
+        <v>13.1</v>
       </c>
       <c r="C3" t="n">
-        <v>1.5</v>
+        <v>1.3</v>
       </c>
       <c r="D3" t="n">
-        <v>83.8</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>0.31</v>
+        <v>0.274</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0113</v>
+        <v>0.0117</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0494</v>
+        <v>0.0479</v>
       </c>
       <c r="H3" t="n">
-        <v>26.9</v>
+        <v>26.2</v>
       </c>
       <c r="I3" t="n">
-        <v>72.5</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="J3" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="4">
@@ -2888,31 +2888,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>5.4</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>93.90000000000001</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="E4" t="n">
-        <v>0.121</v>
+        <v>0.108</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0058</v>
+        <v>0.0056</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0053</v>
+        <v>0.0039</v>
       </c>
       <c r="H4" t="n">
-        <v>36.1</v>
+        <v>37.2</v>
       </c>
       <c r="I4" t="n">
-        <v>63.5</v>
+        <v>62.3</v>
       </c>
       <c r="J4" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="5">
@@ -3049,31 +3049,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6.5</v>
+        <v>5.8</v>
       </c>
       <c r="C12" t="n">
-        <v>1.1</v>
+        <v>0.7</v>
       </c>
       <c r="D12" t="n">
-        <v>92.40000000000001</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>0.141</v>
+        <v>0.124</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.0232</v>
+        <v>-0.0199</v>
       </c>
       <c r="G12" t="n">
-        <v>0.08119999999999999</v>
+        <v>0.0596</v>
       </c>
       <c r="H12" t="n">
-        <v>24</v>
+        <v>23.7</v>
       </c>
       <c r="I12" t="n">
-        <v>75.7</v>
+        <v>76</v>
       </c>
       <c r="J12" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="13">
@@ -3083,28 +3083,28 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2.6</v>
+        <v>2.4</v>
       </c>
       <c r="C13" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>97.2</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>0.054</v>
+        <v>0.048</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.0152</v>
+        <v>-0.0173</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0197</v>
+        <v>0.008</v>
       </c>
       <c r="H13" t="n">
-        <v>40.6</v>
+        <v>39.4</v>
       </c>
       <c r="I13" t="n">
-        <v>59.4</v>
+        <v>60.6</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -3244,31 +3244,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>7.9</v>
+        <v>7</v>
       </c>
       <c r="C21" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>92.90000000000001</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.141</v>
+      </c>
+      <c r="F21" t="n">
+        <v>-0.0039</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.0072</v>
+      </c>
+      <c r="H21" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="I21" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="J21" t="n">
         <v>0.2</v>
-      </c>
-      <c r="D21" t="n">
-        <v>91.90000000000001</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="F21" t="n">
-        <v>-0.0055</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0.0116</v>
-      </c>
-      <c r="H21" t="n">
-        <v>32.7</v>
-      </c>
-      <c r="I21" t="n">
-        <v>67.2</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0.1</v>
       </c>
     </row>
     <row r="22">
@@ -3278,28 +3278,28 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>96.90000000000001</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="E22" t="n">
-        <v>0.061</v>
+        <v>0.057</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.025</v>
+        <v>-0.0224</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0032</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>42.9</v>
+        <v>45</v>
       </c>
       <c r="I22" t="n">
-        <v>57.1</v>
+        <v>55</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
@@ -3439,31 +3439,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>7.6</v>
+        <v>6.6</v>
       </c>
       <c r="C30" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="D30" t="n">
-        <v>91.8</v>
+        <v>92.7</v>
       </c>
       <c r="E30" t="n">
-        <v>0.158</v>
+        <v>0.139</v>
       </c>
       <c r="F30" t="n">
-        <v>0.0238</v>
+        <v>0.0235</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0369</v>
+        <v>0.057</v>
       </c>
       <c r="H30" t="n">
-        <v>28.4</v>
+        <v>28.2</v>
       </c>
       <c r="I30" t="n">
-        <v>71.2</v>
+        <v>71.3</v>
       </c>
       <c r="J30" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="31">
@@ -3473,28 +3473,28 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="C31" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>97.09999999999999</v>
+        <v>97.5</v>
       </c>
       <c r="E31" t="n">
-        <v>0.057</v>
+        <v>0.05</v>
       </c>
       <c r="F31" t="n">
-        <v>0.008</v>
+        <v>0.0053</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0224</v>
+        <v>0.0019</v>
       </c>
       <c r="H31" t="n">
-        <v>35.5</v>
+        <v>34.9</v>
       </c>
       <c r="I31" t="n">
-        <v>64.5</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -3634,28 +3634,28 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>6.1</v>
+        <v>5.7</v>
       </c>
       <c r="C39" t="n">
-        <v>1.8</v>
+        <v>1.1</v>
       </c>
       <c r="D39" t="n">
-        <v>92</v>
+        <v>93.3</v>
       </c>
       <c r="E39" t="n">
-        <v>0.141</v>
+        <v>0.124</v>
       </c>
       <c r="F39" t="n">
-        <v>0.0162</v>
+        <v>0.0145</v>
       </c>
       <c r="G39" t="n">
-        <v>0.13</v>
+        <v>0.0862</v>
       </c>
       <c r="H39" t="n">
-        <v>20.5</v>
+        <v>20</v>
       </c>
       <c r="I39" t="n">
-        <v>79.09999999999999</v>
+        <v>79.7</v>
       </c>
       <c r="J39" t="n">
         <v>0.3</v>
@@ -3668,28 +3668,28 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="C40" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D40" t="n">
-        <v>97.3</v>
+        <v>97.7</v>
       </c>
       <c r="E40" t="n">
-        <v>0.052</v>
+        <v>0.046</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0102</v>
+        <v>0.0078</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0223</v>
+        <v>0.0083</v>
       </c>
       <c r="H40" t="n">
-        <v>39.6</v>
+        <v>38.6</v>
       </c>
       <c r="I40" t="n">
-        <v>60.4</v>
+        <v>61.4</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -3829,31 +3829,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>8.6</v>
+        <v>7.6</v>
       </c>
       <c r="C48" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="D48" t="n">
-        <v>90.40000000000001</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="E48" t="n">
-        <v>0.182</v>
+        <v>0.161</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0045</v>
+        <v>0.0052</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0618</v>
+        <v>0.0516</v>
       </c>
       <c r="H48" t="n">
-        <v>26.7</v>
+        <v>26</v>
       </c>
       <c r="I48" t="n">
-        <v>73</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="J48" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="49">
@@ -3863,31 +3863,31 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>3.4</v>
+        <v>3.1</v>
       </c>
       <c r="C49" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>96.5</v>
+        <v>96.90000000000001</v>
       </c>
       <c r="E49" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.062</v>
       </c>
       <c r="F49" t="n">
-        <v>-0.0032</v>
+        <v>-0.0042</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0146</v>
+        <v>0.0044</v>
       </c>
       <c r="H49" t="n">
-        <v>38.5</v>
+        <v>38.9</v>
       </c>
       <c r="I49" t="n">
-        <v>61.3</v>
+        <v>61</v>
       </c>
       <c r="J49" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="50">
@@ -4038,31 +4038,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7.1</v>
+        <v>4.8</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D3" t="n">
-        <v>92.90000000000001</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="E3" t="n">
-        <v>0.142</v>
+        <v>0.097</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0091</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0024</v>
+        <v>0.0065</v>
       </c>
       <c r="H3" t="n">
-        <v>65.09999999999999</v>
+        <v>62.1</v>
       </c>
       <c r="I3" t="n">
-        <v>33.5</v>
+        <v>33.6</v>
       </c>
       <c r="J3" t="n">
-        <v>1.4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="4">
@@ -4072,31 +4072,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>2.1</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>95.8</v>
+        <v>97.8</v>
       </c>
       <c r="E4" t="n">
-        <v>0.082</v>
+        <v>0.043</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0041</v>
+        <v>-0.0007</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0334</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>73.90000000000001</v>
+        <v>63.9</v>
       </c>
       <c r="I4" t="n">
-        <v>25.1</v>
+        <v>34.5</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="5">
@@ -4233,31 +4233,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4.9</v>
+        <v>3.2</v>
       </c>
       <c r="C12" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="D12" t="n">
-        <v>94.3</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>0.106</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0196</v>
+        <v>0.0235</v>
       </c>
       <c r="G12" t="n">
-        <v>0.07820000000000001</v>
+        <v>0.0612</v>
       </c>
       <c r="H12" t="n">
-        <v>60.1</v>
+        <v>54.4</v>
       </c>
       <c r="I12" t="n">
-        <v>38.5</v>
+        <v>42.1</v>
       </c>
       <c r="J12" t="n">
-        <v>1.4</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="13">
@@ -4267,31 +4267,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2.9</v>
+        <v>1.4</v>
       </c>
       <c r="C13" t="n">
         <v>0.1</v>
       </c>
       <c r="D13" t="n">
-        <v>96.90000000000001</v>
+        <v>98.5</v>
       </c>
       <c r="E13" t="n">
-        <v>0.06</v>
+        <v>0.029</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0026</v>
+        <v>0.014</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0195</v>
+        <v>0.0284</v>
       </c>
       <c r="H13" t="n">
-        <v>70</v>
+        <v>63.4</v>
       </c>
       <c r="I13" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="14">
@@ -4428,31 +4428,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>6.3</v>
+        <v>5</v>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
       <c r="D21" t="n">
-        <v>92.8</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="E21" t="n">
-        <v>0.135</v>
+        <v>0.104</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.0049</v>
+        <v>-0.0071</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0709</v>
+        <v>0.0371</v>
       </c>
       <c r="H21" t="n">
-        <v>70.8</v>
+        <v>64.2</v>
       </c>
       <c r="I21" t="n">
-        <v>27.3</v>
+        <v>32.3</v>
       </c>
       <c r="J21" t="n">
-        <v>1.9</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="22">
@@ -4462,31 +4462,31 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4.2</v>
+        <v>2.6</v>
       </c>
       <c r="C22" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="D22" t="n">
-        <v>95.40000000000001</v>
+        <v>97.3</v>
       </c>
       <c r="E22" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.053</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.018</v>
+        <v>-0.008500000000000001</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0461</v>
+        <v>0.0146</v>
       </c>
       <c r="H22" t="n">
-        <v>76.8</v>
+        <v>72.8</v>
       </c>
       <c r="I22" t="n">
-        <v>21.9</v>
+        <v>25.2</v>
       </c>
       <c r="J22" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
@@ -4623,31 +4623,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>8.300000000000001</v>
+        <v>4.2</v>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D30" t="n">
-        <v>91.7</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="E30" t="n">
-        <v>0.166</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="F30" t="n">
-        <v>0.02</v>
+        <v>0.0171</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0007</v>
+        <v>0.0156</v>
       </c>
       <c r="H30" t="n">
-        <v>53.1</v>
+        <v>47.9</v>
       </c>
       <c r="I30" t="n">
-        <v>45.1</v>
+        <v>45.4</v>
       </c>
       <c r="J30" t="n">
-        <v>1.8</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="31">
@@ -4657,28 +4657,28 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3.1</v>
+        <v>1.3</v>
       </c>
       <c r="C31" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>96.8</v>
+        <v>98.7</v>
       </c>
       <c r="E31" t="n">
-        <v>0.063</v>
+        <v>0.026</v>
       </c>
       <c r="F31" t="n">
-        <v>0.0183</v>
+        <v>-0.0012</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0202</v>
+        <v>0.0035</v>
       </c>
       <c r="H31" t="n">
-        <v>57.5</v>
+        <v>61.1</v>
       </c>
       <c r="I31" t="n">
-        <v>42.5</v>
+        <v>38.9</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -4818,31 +4818,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>5.3</v>
+        <v>3.6</v>
       </c>
       <c r="C39" t="n">
-        <v>0.6</v>
+        <v>0.1</v>
       </c>
       <c r="D39" t="n">
-        <v>94.09999999999999</v>
+        <v>96.3</v>
       </c>
       <c r="E39" t="n">
-        <v>0.113</v>
+        <v>0.073</v>
       </c>
       <c r="F39" t="n">
-        <v>0.0026</v>
+        <v>-0.0019</v>
       </c>
       <c r="G39" t="n">
-        <v>0.0516</v>
+        <v>0.0069</v>
       </c>
       <c r="H39" t="n">
-        <v>51.4</v>
+        <v>46.4</v>
       </c>
       <c r="I39" t="n">
-        <v>46.1</v>
+        <v>47.9</v>
       </c>
       <c r="J39" t="n">
-        <v>2.5</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="40">
@@ -4852,31 +4852,31 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D40" t="n">
-        <v>97</v>
+        <v>98.5</v>
       </c>
       <c r="E40" t="n">
-        <v>0.059</v>
+        <v>0.03</v>
       </c>
       <c r="F40" t="n">
-        <v>-0.0196</v>
+        <v>-0.0161</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0016</v>
+        <v>0.0155</v>
       </c>
       <c r="H40" t="n">
-        <v>65</v>
+        <v>56.3</v>
       </c>
       <c r="I40" t="n">
-        <v>34.2</v>
+        <v>42.7</v>
       </c>
       <c r="J40" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="41">
@@ -5013,31 +5013,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>6.4</v>
+        <v>4.2</v>
       </c>
       <c r="C48" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="D48" t="n">
-        <v>93.09999999999999</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="E48" t="n">
-        <v>0.132</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="F48" t="n">
-        <v>0.009299999999999999</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="G48" t="n">
-        <v>0.0407</v>
+        <v>0.0255</v>
       </c>
       <c r="H48" t="n">
-        <v>60.2</v>
+        <v>55.7</v>
       </c>
       <c r="I48" t="n">
-        <v>38</v>
+        <v>39.5</v>
       </c>
       <c r="J48" t="n">
-        <v>1.8</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="49">
@@ -5047,31 +5047,31 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>3.4</v>
+        <v>1.8</v>
       </c>
       <c r="C49" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="D49" t="n">
-        <v>96.40000000000001</v>
+        <v>98.2</v>
       </c>
       <c r="E49" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.036</v>
       </c>
       <c r="F49" t="n">
-        <v>-0.0041</v>
+        <v>-0.0025</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0242</v>
+        <v>0.0142</v>
       </c>
       <c r="H49" t="n">
-        <v>69.5</v>
+        <v>64.7</v>
       </c>
       <c r="I49" t="n">
-        <v>29.7</v>
+        <v>34</v>
       </c>
       <c r="J49" t="n">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="50">
@@ -5222,31 +5222,31 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.6</v>
+        <v>1.9</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D3" t="n">
-        <v>97.40000000000001</v>
+        <v>98</v>
       </c>
       <c r="E3" t="n">
-        <v>0.051</v>
+        <v>0.038</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.0014</v>
+        <v>-0.014</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0056</v>
+        <v>0.0194</v>
       </c>
       <c r="H3" t="n">
-        <v>52.5</v>
+        <v>49.5</v>
       </c>
       <c r="I3" t="n">
-        <v>34.1</v>
+        <v>26.7</v>
       </c>
       <c r="J3" t="n">
-        <v>13.4</v>
+        <v>23.8</v>
       </c>
     </row>
     <row r="4">
@@ -5256,31 +5256,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.9</v>
+        <v>0.5</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>99.09999999999999</v>
+        <v>99.5</v>
       </c>
       <c r="E4" t="n">
-        <v>0.017</v>
+        <v>0.01</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.0039</v>
+        <v>-0.0194</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0103</v>
+        <v>0.0357</v>
       </c>
       <c r="H4" t="n">
-        <v>58.8</v>
+        <v>55.4</v>
       </c>
       <c r="I4" t="n">
-        <v>38.7</v>
+        <v>40.2</v>
       </c>
       <c r="J4" t="n">
-        <v>2.6</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="5">
@@ -5417,31 +5417,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D12" t="n">
-        <v>99.09999999999999</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>0.018</v>
+        <v>0.012</v>
       </c>
       <c r="F12" t="n">
-        <v>0.005</v>
+        <v>0.0151</v>
       </c>
       <c r="G12" t="n">
-        <v>0.01</v>
+        <v>0.0511</v>
       </c>
       <c r="H12" t="n">
-        <v>42</v>
+        <v>40.1</v>
       </c>
       <c r="I12" t="n">
-        <v>39</v>
+        <v>31.4</v>
       </c>
       <c r="J12" t="n">
-        <v>19</v>
+        <v>28.5</v>
       </c>
     </row>
     <row r="13">
@@ -5451,28 +5451,28 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>99.8</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="E13" t="n">
-        <v>0.005</v>
+        <v>0.002</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0115</v>
+        <v>0.015</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>57.4</v>
+        <v>42.9</v>
       </c>
       <c r="I13" t="n">
-        <v>42.6</v>
+        <v>57.1</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -5612,31 +5612,31 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="C21" t="n">
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>99</v>
+        <v>99.2</v>
       </c>
       <c r="E21" t="n">
-        <v>0.021</v>
+        <v>0.015</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.012</v>
+        <v>-0.0165</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0131</v>
+        <v>0.0289</v>
       </c>
       <c r="H21" t="n">
-        <v>44.1</v>
+        <v>40.5</v>
       </c>
       <c r="I21" t="n">
-        <v>37.6</v>
+        <v>28.3</v>
       </c>
       <c r="J21" t="n">
-        <v>18.3</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="22">
@@ -5646,31 +5646,31 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="C22" t="n">
         <v>0</v>
       </c>
       <c r="D22" t="n">
-        <v>99.7</v>
+        <v>99.8</v>
       </c>
       <c r="E22" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
       <c r="F22" t="n">
-        <v>-0.0075</v>
+        <v>-0.0294</v>
       </c>
       <c r="G22" t="n">
-        <v>0.0159</v>
+        <v>0.0556</v>
       </c>
       <c r="H22" t="n">
-        <v>49.2</v>
+        <v>72.2</v>
       </c>
       <c r="I22" t="n">
-        <v>49.2</v>
+        <v>27.8</v>
       </c>
       <c r="J22" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -5807,31 +5807,31 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="C30" t="n">
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>99</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E30" t="n">
-        <v>0.02</v>
+        <v>0.013</v>
       </c>
       <c r="F30" t="n">
-        <v>0.0067</v>
+        <v>0.0094</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0046</v>
+        <v>0.0068</v>
       </c>
       <c r="H30" t="n">
-        <v>48.4</v>
+        <v>42.2</v>
       </c>
       <c r="I30" t="n">
-        <v>38.8</v>
+        <v>34</v>
       </c>
       <c r="J30" t="n">
-        <v>12.8</v>
+        <v>23.8</v>
       </c>
     </row>
     <row r="31">
@@ -5841,28 +5841,28 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="C31" t="n">
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>99.7</v>
+        <v>99.8</v>
       </c>
       <c r="E31" t="n">
-        <v>0.007</v>
+        <v>0.003</v>
       </c>
       <c r="F31" t="n">
-        <v>0.0032</v>
+        <v>0.0273</v>
       </c>
       <c r="G31" t="n">
-        <v>0.0127</v>
+        <v>0.0256</v>
       </c>
       <c r="H31" t="n">
-        <v>69.59999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="I31" t="n">
-        <v>30.4</v>
+        <v>30.8</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -6002,31 +6002,31 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="C39" t="n">
         <v>0.1</v>
       </c>
       <c r="D39" t="n">
-        <v>99</v>
+        <v>99.3</v>
       </c>
       <c r="E39" t="n">
-        <v>0.019</v>
+        <v>0.013</v>
       </c>
       <c r="F39" t="n">
-        <v>0.0151</v>
+        <v>0.0324</v>
       </c>
       <c r="G39" t="n">
-        <v>0.0419</v>
+        <v>0.0621</v>
       </c>
       <c r="H39" t="n">
-        <v>49.3</v>
+        <v>51.7</v>
       </c>
       <c r="I39" t="n">
-        <v>36.7</v>
+        <v>23.4</v>
       </c>
       <c r="J39" t="n">
-        <v>14</v>
+        <v>24.8</v>
       </c>
     </row>
     <row r="40">
@@ -6036,10 +6036,10 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D40" t="n">
         <v>99.8</v>
@@ -6048,19 +6048,19 @@
         <v>0.004</v>
       </c>
       <c r="F40" t="n">
-        <v>0.0054</v>
+        <v>-0.0038</v>
       </c>
       <c r="G40" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.1707</v>
       </c>
       <c r="H40" t="n">
-        <v>84.8</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="I40" t="n">
-        <v>13</v>
+        <v>12.2</v>
       </c>
       <c r="J40" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="41">
@@ -6197,31 +6197,31 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1.3</v>
+        <v>0.9</v>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D48" t="n">
-        <v>98.7</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="E48" t="n">
-        <v>0.026</v>
+        <v>0.018</v>
       </c>
       <c r="F48" t="n">
-        <v>0.0027</v>
+        <v>0.0053</v>
       </c>
       <c r="G48" t="n">
-        <v>0.015</v>
+        <v>0.0337</v>
       </c>
       <c r="H48" t="n">
-        <v>48.5</v>
+        <v>46</v>
       </c>
       <c r="I48" t="n">
-        <v>36.5</v>
+        <v>28.2</v>
       </c>
       <c r="J48" t="n">
-        <v>15</v>
+        <v>25.8</v>
       </c>
     </row>
     <row r="49">
@@ -6231,31 +6231,31 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="C49" t="n">
         <v>0</v>
       </c>
       <c r="D49" t="n">
-        <v>99.59999999999999</v>
+        <v>99.8</v>
       </c>
       <c r="E49" t="n">
-        <v>0.008</v>
+        <v>0.004</v>
       </c>
       <c r="F49" t="n">
-        <v>0.0017</v>
+        <v>-0.0021</v>
       </c>
       <c r="G49" t="n">
-        <v>0.0252</v>
+        <v>0.0575</v>
       </c>
       <c r="H49" t="n">
-        <v>61.9</v>
+        <v>63.3</v>
       </c>
       <c r="I49" t="n">
-        <v>36.5</v>
+        <v>34.4</v>
       </c>
       <c r="J49" t="n">
-        <v>1.6</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="50">

</xml_diff>